<commit_message>
Auto-collected traffic data: 2026-09-03 02:54 AM IST [12_00 AM]
</commit_message>
<xml_diff>
--- a/output/excel/Kolkata_Traffic_Data_2026-09-03.xlsx
+++ b/output/excel/Kolkata_Traffic_Data_2026-09-03.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="408">
   <si>
     <t>Route ID</t>
   </si>
@@ -106,10 +106,13 @@
     <t>19.7 km</t>
   </si>
   <si>
-    <t>26.3</t>
-  </si>
-  <si>
-    <t>Equal</t>
+    <t>26.9</t>
+  </si>
+  <si>
+    <t>28.1</t>
+  </si>
+  <si>
+    <t>-2 min (Bike Faster)</t>
   </si>
   <si>
     <t>17.1</t>
@@ -123,7 +126,7 @@
 AC-52</t>
   </si>
   <si>
-    <t>1.53x</t>
+    <t>1.57x</t>
   </si>
   <si>
     <t>Walk: 0 min</t>
@@ -150,13 +153,13 @@
     <t>6.0 km</t>
   </si>
   <si>
-    <t>27.7</t>
+    <t>32.7</t>
   </si>
   <si>
     <t>30.0</t>
   </si>
   <si>
-    <t>-1 min (Bike Faster)</t>
+    <t>+1 min (Car Faster)</t>
   </si>
   <si>
     <t xml:space="preserve">21 min
@@ -166,7 +169,7 @@
 Details</t>
   </si>
   <si>
-    <t>1.62x</t>
+    <t>1.91x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M02_B_T_Road/car.jpg</t>
@@ -187,11 +190,14 @@
     <t>38.8</t>
   </si>
   <si>
+    <t>Equal</t>
+  </si>
+  <si>
     <t>17.2</t>
   </si>
   <si>
     <t xml:space="preserve">43 min
-2:09 AM (Wednesday)—2:52 AM
+5:09 AM (Wednesday)—5:52 AM
 78</t>
   </si>
   <si>
@@ -216,13 +222,7 @@
     <t>14.9 km</t>
   </si>
   <si>
-    <t>34.4</t>
-  </si>
-  <si>
     <t>37.3</t>
-  </si>
-  <si>
-    <t>-2 min (Bike Faster)</t>
   </si>
   <si>
     <t>22.4</t>
@@ -233,7 +233,7 @@
 217  </t>
   </si>
   <si>
-    <t>1.54x</t>
+    <t>1.67x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M04_VIP_Road/car.jpg</t>
@@ -254,10 +254,10 @@
     <t>11.3 km</t>
   </si>
   <si>
-    <t>19.4</t>
-  </si>
-  <si>
-    <t>26.1</t>
+    <t>18.8</t>
+  </si>
+  <si>
+    <t>25.1</t>
   </si>
   <si>
     <t>-9 min (Bike Faster)</t>
@@ -273,7 +273,7 @@
 Details</t>
   </si>
   <si>
-    <t>1.11x</t>
+    <t>1.08x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M05_Jessore_Road/car.jpg</t>
@@ -294,10 +294,10 @@
     <t>4.8 km</t>
   </si>
   <si>
+    <t>32.0</t>
+  </si>
+  <si>
     <t>28.8</t>
-  </si>
-  <si>
-    <t>32.0</t>
   </si>
   <si>
     <t>2.7</t>
@@ -314,7 +314,7 @@
 Details</t>
   </si>
   <si>
-    <t>10.70x</t>
+    <t>11.89x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M06_Airport_Road/car.jpg</t>
@@ -335,10 +335,13 @@
     <t>8.2 km</t>
   </si>
   <si>
-    <t>21.4</t>
-  </si>
-  <si>
     <t>23.4</t>
+  </si>
+  <si>
+    <t>24.6</t>
+  </si>
+  <si>
+    <t>-1 min (Bike Faster)</t>
   </si>
   <si>
     <t>17.0</t>
@@ -351,7 +354,7 @@
 Details</t>
   </si>
   <si>
-    <t>1.26x</t>
+    <t>1.38x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M07_APC_Bose_Rd/car.jpg</t>
@@ -369,7 +372,7 @@
     <t>Bidhan Sarani</t>
   </si>
   <si>
-    <t>25.7</t>
+    <t>27.7</t>
   </si>
   <si>
     <t>16.4</t>
@@ -380,7 +383,7 @@
 34B</t>
   </si>
   <si>
-    <t>1.57x</t>
+    <t>1.69x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M08_Bidhan_Sarani/car.jpg</t>
@@ -401,7 +404,7 @@
     <t>5.0 km</t>
   </si>
   <si>
-    <t>20.0</t>
+    <t>21.4</t>
   </si>
   <si>
     <t>23.1</t>
@@ -415,7 +418,7 @@
   34B</t>
   </si>
   <si>
-    <t>1.60x</t>
+    <t>1.71x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M09_Central_Avenue__C_R_Avenue_/car.jpg</t>
@@ -437,6 +440,9 @@
   </si>
   <si>
     <t>23.0</t>
+  </si>
+  <si>
+    <t>27.6</t>
   </si>
   <si>
     <t>19.7</t>
@@ -468,7 +474,13 @@
     <t>4.2 km</t>
   </si>
   <si>
+    <t>28.0</t>
+  </si>
+  <si>
     <t>25.2</t>
+  </si>
+  <si>
+    <t>19.4</t>
   </si>
   <si>
     <t xml:space="preserve">13 min
@@ -476,7 +488,7 @@
 28</t>
   </si>
   <si>
-    <t>1.30x</t>
+    <t>1.44x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M11_M_G_Road/car.jpg</t>
@@ -495,9 +507,6 @@
   </si>
   <si>
     <t>2.6 km</t>
-  </si>
-  <si>
-    <t>22.3</t>
   </si>
   <si>
     <t>26.0</t>
@@ -511,7 +520,7 @@
 45</t>
   </si>
   <si>
-    <t>1.29x</t>
+    <t>1.50x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M12_C_I_T_Road/car.jpg</t>
@@ -532,10 +541,10 @@
     <t>3.8 km</t>
   </si>
   <si>
-    <t>22.8</t>
-  </si>
-  <si>
     <t>25.3</t>
+  </si>
+  <si>
+    <t>28.5</t>
   </si>
   <si>
     <t>17.5</t>
@@ -564,7 +573,10 @@
     <t>15.6 km</t>
   </si>
   <si>
-    <t>24.6</t>
+    <t>27.5</t>
+  </si>
+  <si>
+    <t>28.4</t>
   </si>
   <si>
     <t>14.4</t>
@@ -573,9 +585,6 @@
     <t xml:space="preserve">1 hr 5 min
 2:01 AM (Wednesday)—3:06 AM
 46B  45</t>
-  </si>
-  <si>
-    <t>1.63x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M14_S_P_Mukherjee_Road/car.jpg</t>
@@ -628,7 +637,7 @@
     <t>2.9 km</t>
   </si>
   <si>
-    <t>24.9</t>
+    <t>29.0</t>
   </si>
   <si>
     <t>8.3</t>
@@ -639,7 +648,7 @@
 1  </t>
   </si>
   <si>
-    <t>3.00x</t>
+    <t>3.50x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M16_Gariahat_Road___Rashbehari_Avenue/car.jpg</t>
@@ -658,12 +667,6 @@
   </si>
   <si>
     <t>2.8 km</t>
-  </si>
-  <si>
-    <t>24.0</t>
-  </si>
-  <si>
-    <t>28.0</t>
   </si>
   <si>
     <t>8.0</t>
@@ -692,6 +695,9 @@
     <t>3.9 km</t>
   </si>
   <si>
+    <t>29.3</t>
+  </si>
+  <si>
     <t>6.5</t>
   </si>
   <si>
@@ -700,7 +706,7 @@
   234/1  S-131</t>
   </si>
   <si>
-    <t>3.60x</t>
+    <t>4.00x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M19_Taratala_Road/car.jpg</t>
@@ -721,7 +727,7 @@
     <t>6.9 km</t>
   </si>
   <si>
-    <t>25.9</t>
+    <t>29.6</t>
   </si>
   <si>
     <t>5.2</t>
@@ -732,7 +738,7 @@
   1B  </t>
   </si>
   <si>
-    <t>5.00x</t>
+    <t>5.71x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M20_Prince_Anwar_Shah_Rd/car.jpg</t>
@@ -780,7 +786,7 @@
     <t>5.5 km</t>
   </si>
   <si>
-    <t>27.5</t>
+    <t>33.0</t>
   </si>
   <si>
     <t>9.2</t>
@@ -794,6 +800,9 @@
 Details</t>
   </si>
   <si>
+    <t>3.60x</t>
+  </si>
+  <si>
     <t>screenshots/2026-09-03/12_00 AM/M22_Canal_South_Road/car.jpg</t>
   </si>
   <si>
@@ -810,6 +819,9 @@
   </si>
   <si>
     <t>4.1 km</t>
+  </si>
+  <si>
+    <t>27.3</t>
   </si>
   <si>
     <t>12.3</t>
@@ -820,7 +832,7 @@
 201  </t>
   </si>
   <si>
-    <t>2.00x</t>
+    <t>2.22x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/M23_VIP_Road_connector/car.jpg</t>
@@ -855,6 +867,9 @@
 45</t>
   </si>
   <si>
+    <t>2.00x</t>
+  </si>
+  <si>
     <t>screenshots/2026-09-03/12_00 AM/S01_Baishnabghata_Patuli/car.jpg</t>
   </si>
   <si>
@@ -915,6 +930,9 @@
     <t>1.7 km</t>
   </si>
   <si>
+    <t>34.0</t>
+  </si>
+  <si>
     <t>screenshots/2026-09-03/12_00 AM/S04_Ajaynagar___Kalikapur/car.jpg</t>
   </si>
   <si>
@@ -954,6 +972,9 @@
     <t>4.0 km</t>
   </si>
   <si>
+    <t>40.0</t>
+  </si>
+  <si>
     <t>34.3</t>
   </si>
   <si>
@@ -993,7 +1014,7 @@
     <t>Chingrighata - Sealdah</t>
   </si>
   <si>
-    <t>30.7</t>
+    <t>34.5</t>
   </si>
   <si>
     <t>18.4</t>
@@ -1004,7 +1025,7 @@
 S-12N</t>
   </si>
   <si>
-    <t>1.67x</t>
+    <t>1.88x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/S08_Chingrighata___Sealdah/car.jpg</t>
@@ -1020,6 +1041,9 @@
   </si>
   <si>
     <t>Sealdah - Park Circus</t>
+  </si>
+  <si>
+    <t>24.9</t>
   </si>
   <si>
     <t>3.9</t>
@@ -1030,7 +1054,7 @@
 S-12N  230  </t>
   </si>
   <si>
-    <t>6.43x</t>
+    <t>7.50x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/S09_Sealdah___Park_Circus/car.jpg</t>
@@ -1049,9 +1073,6 @@
   </si>
   <si>
     <t>45.6</t>
-  </si>
-  <si>
-    <t>+1 min (Car Faster)</t>
   </si>
   <si>
     <t>12.0</t>
@@ -1083,7 +1104,7 @@
     <t>2.7 km</t>
   </si>
   <si>
-    <t>27.0</t>
+    <t>32.4</t>
   </si>
   <si>
     <t>13.5</t>
@@ -1094,7 +1115,7 @@
 45</t>
   </si>
   <si>
-    <t>1.71x</t>
+    <t>2.40x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/S11_Park_Circus___Gariahat/car.jpg</t>
@@ -1112,7 +1133,7 @@
     <t>Gariahat - Ruby</t>
   </si>
   <si>
-    <t>27.3</t>
+    <t>30.7</t>
   </si>
   <si>
     <t>17.6</t>
@@ -1123,7 +1144,7 @@
 18B/1</t>
   </si>
   <si>
-    <t>1.56x</t>
+    <t>1.75x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/S12_Gariahat___Ruby/car.jpg</t>
@@ -1149,9 +1170,6 @@
 45</t>
   </si>
   <si>
-    <t>1.75x</t>
-  </si>
-  <si>
     <t>screenshots/2026-09-03/12_00 AM/S13_Gariahat___Mallick_Road/car.jpg</t>
   </si>
   <si>
@@ -1168,6 +1186,9 @@
   </si>
   <si>
     <t>3.5 km</t>
+  </si>
+  <si>
+    <t>35.0</t>
   </si>
   <si>
     <t>5.0</t>
@@ -1178,7 +1199,7 @@
 1B  </t>
   </si>
   <si>
-    <t>6.00x</t>
+    <t>7.00x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/S14_Jadavpur_Police_St____Kalikapur/car.jpg</t>
@@ -1206,9 +1227,6 @@
 Details</t>
   </si>
   <si>
-    <t>1.33x</t>
-  </si>
-  <si>
     <t>screenshots/2026-09-03/12_00 AM/S15_Mallick_Road___Jadavpur_Sulekha/car.jpg</t>
   </si>
   <si>
@@ -1225,6 +1243,9 @@
   </si>
   <si>
     <t>3.1 km</t>
+  </si>
+  <si>
+    <t>31.0</t>
   </si>
   <si>
     <t>26.6</t>
@@ -1238,9 +1259,6 @@
 S-9</t>
   </si>
   <si>
-    <t>1.43x</t>
-  </si>
-  <si>
     <t>screenshots/2026-09-03/12_00 AM/S16_Jadavpur_Sulekha___Ajay_Nagar/car.jpg</t>
   </si>
   <si>
@@ -1257,6 +1275,9 @@
   </si>
   <si>
     <t>900 m</t>
+  </si>
+  <si>
+    <t>27.0</t>
   </si>
   <si>
     <t>18.0</t>
@@ -1265,9 +1286,6 @@
     <t xml:space="preserve">3 min
 5:58 AM (Wednesday)—6:01 AM
 13C</t>
-  </si>
-  <si>
-    <t>1.50x</t>
   </si>
   <si>
     <t>screenshots/2026-09-03/12_00 AM/S17_Jadavpur_Sulekha___Bagha_Jatin/car.jpg</t>
@@ -1886,7 +1904,7 @@
         <v>30</v>
       </c>
       <c r="G2" s="5">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>31</v>
@@ -1895,13 +1913,13 @@
         <v>30</v>
       </c>
       <c r="J2" s="2">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>30</v>
@@ -1916,42 +1934,42 @@
         <v>0</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Y2" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>28</v>
@@ -1960,28 +1978,28 @@
         <v>29</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="6">
-        <v>13</v>
+        <v>45</v>
+      </c>
+      <c r="G3" s="9">
+        <v>11</v>
       </c>
       <c r="H3" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>45</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>44</v>
       </c>
       <c r="J3" s="6">
         <v>12</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N3" s="6">
         <v>21</v>
@@ -1993,42 +2011,42 @@
         <v>0</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R3" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S3" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T3" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U3" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V3" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W3" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="X3" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y3" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>28</v>
@@ -2037,28 +2055,28 @@
         <v>29</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G4" s="2">
+        <v>55</v>
+      </c>
+      <c r="G4" s="5">
         <v>19</v>
       </c>
       <c r="H4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>54</v>
       </c>
       <c r="J4" s="2">
         <v>19</v>
       </c>
       <c r="K4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>54</v>
       </c>
       <c r="N4" s="2">
         <v>43</v>
@@ -2070,42 +2088,42 @@
         <v>0</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="X4" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Y4" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>28</v>
@@ -2114,28 +2132,28 @@
         <v>29</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G5" s="6">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J5" s="6">
         <v>24</v>
       </c>
       <c r="K5" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="M5" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>64</v>
       </c>
       <c r="N5" s="6">
         <v>40</v>
@@ -2150,7 +2168,7 @@
         <v>68</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S5" s="7" t="s">
         <v>69</v>
@@ -2159,10 +2177,10 @@
         <v>70</v>
       </c>
       <c r="U5" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V5" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W5" s="7" t="s">
         <v>71</v>
@@ -2194,7 +2212,7 @@
         <v>76</v>
       </c>
       <c r="G6" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>77</v>
@@ -2203,7 +2221,7 @@
         <v>76</v>
       </c>
       <c r="J6" s="2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>78</v>
@@ -2227,7 +2245,7 @@
         <v>80</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S6" s="3" t="s">
         <v>81</v>
@@ -2236,10 +2254,10 @@
         <v>82</v>
       </c>
       <c r="U6" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V6" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W6" s="3" t="s">
         <v>83</v>
@@ -2271,7 +2289,7 @@
         <v>88</v>
       </c>
       <c r="G7" s="9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>89</v>
@@ -2280,13 +2298,13 @@
         <v>88</v>
       </c>
       <c r="J7" s="6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>90</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M7" s="7" t="s">
         <v>88</v>
@@ -2313,10 +2331,10 @@
         <v>94</v>
       </c>
       <c r="U7" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V7" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W7" s="7" t="s">
         <v>95</v>
@@ -2348,7 +2366,7 @@
         <v>100</v>
       </c>
       <c r="G8" s="5">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>101</v>
@@ -2357,13 +2375,13 @@
         <v>100</v>
       </c>
       <c r="J8" s="2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>102</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>67</v>
+        <v>103</v>
       </c>
       <c r="M8" s="3" t="s">
         <v>100</v>
@@ -2378,42 +2396,42 @@
         <v>0</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U8" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V8" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W8" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="X8" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Y8" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>28</v>
@@ -2422,28 +2440,28 @@
         <v>29</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G9" s="9">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J9" s="6">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N9" s="6">
         <v>22</v>
@@ -2455,42 +2473,42 @@
         <v>0</v>
       </c>
       <c r="Q9" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S9" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="T9" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="U9" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V9" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W9" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X9" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Y9" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>28</v>
@@ -2499,28 +2517,28 @@
         <v>29</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G10" s="5">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H10" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>121</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>120</v>
       </c>
       <c r="J10" s="2">
         <v>13</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>67</v>
+        <v>103</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N10" s="2">
         <v>24</v>
@@ -2532,42 +2550,42 @@
         <v>0</v>
       </c>
       <c r="Q10" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="R10" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="U10" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V10" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W10" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="X10" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Y10" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>28</v>
@@ -2576,28 +2594,28 @@
         <v>29</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G11" s="9">
         <v>6</v>
       </c>
       <c r="H11" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I11" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="I11" s="7" t="s">
-        <v>131</v>
-      </c>
       <c r="J11" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K11" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M11" s="7" t="s">
         <v>132</v>
-      </c>
-      <c r="L11" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="M11" s="7" t="s">
-        <v>131</v>
       </c>
       <c r="N11" s="6">
         <v>7</v>
@@ -2609,42 +2627,42 @@
         <v>0</v>
       </c>
       <c r="Q11" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="R11" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S11" s="7" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="T11" s="7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="U11" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V11" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W11" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="X11" s="7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="Y11" s="7" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>28</v>
@@ -2653,28 +2671,28 @@
         <v>29</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="G12" s="2">
-        <v>10</v>
+        <v>143</v>
+      </c>
+      <c r="G12" s="5">
+        <v>9</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J12" s="2">
         <v>10</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="N12" s="2">
         <v>13</v>
@@ -2686,42 +2704,42 @@
         <v>0</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>77</v>
+        <v>146</v>
       </c>
       <c r="R12" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="T12" s="3" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="U12" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V12" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="X12" s="3" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="Y12" s="3" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>28</v>
@@ -2730,28 +2748,28 @@
         <v>29</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G13" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="J13" s="6">
         <v>6</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="N13" s="6">
         <v>9</v>
@@ -2763,42 +2781,42 @@
         <v>0</v>
       </c>
       <c r="Q13" s="7" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R13" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S13" s="7" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="T13" s="7" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="U13" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V13" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W13" s="7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="X13" s="7" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="Y13" s="7" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>28</v>
@@ -2807,28 +2825,28 @@
         <v>29</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="G14" s="5">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="J14" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>47</v>
+        <v>103</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="N14" s="2">
         <v>13</v>
@@ -2840,42 +2858,42 @@
         <v>0</v>
       </c>
       <c r="Q14" s="3" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="R14" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S14" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="T14" s="3" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="U14" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V14" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W14" s="3" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="X14" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="Y14" s="3" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>28</v>
@@ -2884,28 +2902,28 @@
         <v>29</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="G15" s="9">
-        <v>40</v>
+        <v>174</v>
+      </c>
+      <c r="G15" s="6">
+        <v>34</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>102</v>
+        <v>175</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="J15" s="6">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>67</v>
+        <v>103</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="N15" s="6">
         <v>65</v>
@@ -2917,42 +2935,42 @@
         <v>0</v>
       </c>
       <c r="Q15" s="7" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="R15" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S15" s="7" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="T15" s="7" t="s">
-        <v>175</v>
+        <v>50</v>
       </c>
       <c r="U15" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V15" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W15" s="7" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="X15" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="Y15" s="7" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>28</v>
@@ -2961,28 +2979,28 @@
         <v>29</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="G16" s="5">
         <v>12</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="J16" s="2">
         <v>12</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="N16" s="2">
         <v>28</v>
@@ -2994,42 +3012,42 @@
         <v>0</v>
       </c>
       <c r="Q16" s="3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="R16" s="3" t="s">
         <v>92</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="T16" s="3" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="U16" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V16" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W16" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="X16" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="Y16" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>28</v>
@@ -3038,28 +3056,28 @@
         <v>29</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="G17" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="J17" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="N17" s="6">
         <v>21</v>
@@ -3071,42 +3089,42 @@
         <v>0</v>
       </c>
       <c r="Q17" s="7" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="R17" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S17" s="7" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="T17" s="7" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="U17" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V17" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W17" s="7" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="X17" s="7" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="Y17" s="7" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>28</v>
@@ -3115,28 +3133,28 @@
         <v>29</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="G18" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>201</v>
+        <v>144</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="J18" s="2">
         <v>6</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>202</v>
+        <v>144</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="N18" s="2">
         <v>21</v>
@@ -3148,42 +3166,42 @@
         <v>0</v>
       </c>
       <c r="Q18" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="R18" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S18" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="T18" s="3" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="U18" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V18" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W18" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="X18" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Y18" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>28</v>
@@ -3192,28 +3210,28 @@
         <v>29</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G19" s="9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>102</v>
+        <v>155</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J19" s="6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>152</v>
+        <v>212</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>47</v>
+        <v>103</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="N19" s="6">
         <v>36</v>
@@ -3225,42 +3243,42 @@
         <v>0</v>
       </c>
       <c r="Q19" s="7" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="R19" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S19" s="7" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="T19" s="7" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="U19" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V19" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W19" s="7" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="X19" s="7" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="Y19" s="7" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>28</v>
@@ -3269,28 +3287,28 @@
         <v>29</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G20" s="5">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="J20" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="N20" s="2">
         <v>80</v>
@@ -3302,42 +3320,42 @@
         <v>0</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="R20" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="T20" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="U20" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V20" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W20" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="X20" s="3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="Y20" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>28</v>
@@ -3346,75 +3364,75 @@
         <v>29</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="G21" s="9">
         <v>7</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="J21" s="6">
         <v>7</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="N21" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O21" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P21" s="6">
         <v>0</v>
       </c>
       <c r="Q21" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="R21" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="S21" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="T21" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="U21" s="7" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="V21" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W21" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="X21" s="7" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="Y21" s="7" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>28</v>
@@ -3423,28 +3441,28 @@
         <v>29</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G22" s="5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="J22" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>46</v>
+        <v>241</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="N22" s="2">
         <v>36</v>
@@ -3456,42 +3474,42 @@
         <v>0</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="R22" s="3" t="s">
         <v>92</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="T22" s="3" t="s">
-        <v>194</v>
+        <v>244</v>
       </c>
       <c r="U22" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V22" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W22" s="3" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="X22" s="3" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="Y22" s="3" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>28</v>
@@ -3500,28 +3518,28 @@
         <v>29</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="G23" s="9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>172</v>
+        <v>251</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="J23" s="6">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>172</v>
+        <v>251</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M23" s="7" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="N23" s="6">
         <v>20</v>
@@ -3533,42 +3551,42 @@
         <v>0</v>
       </c>
       <c r="Q23" s="7" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="R23" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S23" s="7" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="T23" s="7" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="U23" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V23" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W23" s="7" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="X23" s="7" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="Y23" s="7" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>28</v>
@@ -3577,28 +3595,28 @@
         <v>29</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="G24" s="5">
         <v>4</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="J24" s="2">
         <v>4</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="N24" s="2">
         <v>8</v>
@@ -3610,42 +3628,42 @@
         <v>0</v>
       </c>
       <c r="Q24" s="3" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="R24" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="T24" s="3" t="s">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="U24" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V24" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W24" s="3" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="X24" s="3" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="Y24" s="3" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>28</v>
@@ -3654,75 +3672,75 @@
         <v>29</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="G25" s="9">
         <v>2</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="J25" s="6">
         <v>2</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="N25" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O25" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P25" s="6">
         <v>0</v>
       </c>
       <c r="Q25" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="R25" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="S25" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="T25" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="U25" s="7" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="V25" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W25" s="7" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="X25" s="7" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="Y25" s="7" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>28</v>
@@ -3731,75 +3749,75 @@
         <v>29</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="G26" s="5">
         <v>2</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="J26" s="2">
         <v>2</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P26" s="2">
         <v>0</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="R26" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="S26" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="T26" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="U26" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="V26" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W26" s="3" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="X26" s="3" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="Y26" s="3" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>28</v>
@@ -3808,75 +3826,75 @@
         <v>29</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="G27" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="J27" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M27" s="7" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="N27" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O27" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P27" s="6">
         <v>0</v>
       </c>
       <c r="Q27" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="R27" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="S27" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="T27" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="U27" s="7" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="V27" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W27" s="7" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="X27" s="7" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="Y27" s="7" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>28</v>
@@ -3885,75 +3903,75 @@
         <v>29</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="G28" s="5">
         <v>2</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="J28" s="2">
         <v>2</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P28" s="2">
         <v>0</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="R28" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="S28" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="T28" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="U28" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="V28" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W28" s="3" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="X28" s="3" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="Y28" s="3" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>28</v>
@@ -3962,75 +3980,75 @@
         <v>29</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="G29" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="J29" s="6">
         <v>7</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="N29" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O29" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P29" s="6">
         <v>0</v>
       </c>
       <c r="Q29" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="R29" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="S29" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="T29" s="7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="U29" s="7" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="V29" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W29" s="7" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="X29" s="7" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="Y29" s="7" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>28</v>
@@ -4039,75 +4057,75 @@
         <v>29</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="G30" s="5">
         <v>3</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="J30" s="2">
         <v>3</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P30" s="2">
         <v>0</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="R30" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="T30" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="U30" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="V30" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W30" s="3" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="X30" s="3" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="Y30" s="3" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="D31" s="8" t="s">
         <v>28</v>
@@ -4116,28 +4134,28 @@
         <v>29</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="G31" s="9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="J31" s="6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M31" s="7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="N31" s="6">
         <v>15</v>
@@ -4149,42 +4167,42 @@
         <v>0</v>
       </c>
       <c r="Q31" s="7" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="R31" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S31" s="7" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="T31" s="7" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="U31" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V31" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W31" s="7" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="X31" s="7" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="Y31" s="7" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>28</v>
@@ -4193,28 +4211,28 @@
         <v>29</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="G32" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="J32" s="2">
         <v>7</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>191</v>
+        <v>323</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="M32" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="N32" s="2">
         <v>45</v>
@@ -4226,42 +4244,42 @@
         <v>0</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="T32" s="3" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="U32" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V32" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W32" s="3" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="X32" s="3" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="Y32" s="3" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>28</v>
@@ -4270,28 +4288,28 @@
         <v>29</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="G33" s="9">
         <v>5</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="J33" s="6">
         <v>6</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>325</v>
+        <v>48</v>
       </c>
       <c r="M33" s="7" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="N33" s="6">
         <v>19</v>
@@ -4303,42 +4321,42 @@
         <v>0</v>
       </c>
       <c r="Q33" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="R33" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S33" s="7" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="T33" s="7" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="U33" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V33" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W33" s="7" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="X33" s="7" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="Y33" s="7" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>28</v>
@@ -4347,28 +4365,28 @@
         <v>29</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="G34" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>122</v>
+        <v>342</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="J34" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="N34" s="2">
         <v>12</v>
@@ -4380,42 +4398,42 @@
         <v>0</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="T34" s="3" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="U34" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V34" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W34" s="3" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="X34" s="3" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="Y34" s="3" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D35" s="8" t="s">
         <v>28</v>
@@ -4424,28 +4442,28 @@
         <v>29</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="G35" s="9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="J35" s="6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M35" s="7" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="N35" s="6">
         <v>14</v>
@@ -4457,42 +4475,42 @@
         <v>0</v>
       </c>
       <c r="Q35" s="7" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="R35" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S35" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="T35" s="7" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="U35" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V35" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W35" s="7" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="X35" s="7" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="Y35" s="7" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>28</v>
@@ -4501,28 +4519,28 @@
         <v>29</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="G36" s="5">
         <v>4</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="J36" s="2">
         <v>4</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M36" s="3" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="N36" s="2">
         <v>7</v>
@@ -4534,42 +4552,42 @@
         <v>0</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R36" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S36" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="T36" s="3" t="s">
         <v>354</v>
       </c>
-      <c r="T36" s="3" t="s">
-        <v>355</v>
-      </c>
       <c r="U36" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V36" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W36" s="3" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="X36" s="3" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="Y36" s="3" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="D37" s="8" t="s">
         <v>28</v>
@@ -4578,28 +4596,28 @@
         <v>29</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="G37" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>46</v>
+        <v>368</v>
       </c>
       <c r="I37" s="7" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="J37" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>46</v>
+        <v>368</v>
       </c>
       <c r="L37" s="7" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M37" s="7" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="N37" s="6">
         <v>42</v>
@@ -4611,42 +4629,42 @@
         <v>0</v>
       </c>
       <c r="Q37" s="7" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="R37" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S37" s="7" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="T37" s="7" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="U37" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V37" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W37" s="7" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="X37" s="7" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="Y37" s="7" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>28</v>
@@ -4655,28 +4673,28 @@
         <v>29</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="G38" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>152</v>
+        <v>272</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="J38" s="2">
         <v>2</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="M38" s="3" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="N38" s="2">
         <v>4</v>
@@ -4688,42 +4706,42 @@
         <v>0</v>
       </c>
       <c r="Q38" s="3" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="R38" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S38" s="3" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="T38" s="3" t="s">
-        <v>372</v>
+        <v>265</v>
       </c>
       <c r="U38" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V38" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W38" s="3" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="X38" s="3" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="Y38" s="3" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="D39" s="8" t="s">
         <v>28</v>
@@ -4732,28 +4750,28 @@
         <v>29</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="G39" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="I39" s="7" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="J39" s="6">
         <v>7</v>
       </c>
       <c r="K39" s="7" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="L39" s="7" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="M39" s="7" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="N39" s="6">
         <v>10</v>
@@ -4765,42 +4783,42 @@
         <v>0</v>
       </c>
       <c r="Q39" s="7" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="R39" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S39" s="7" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="T39" s="7" t="s">
-        <v>382</v>
+        <v>70</v>
       </c>
       <c r="U39" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V39" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W39" s="7" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="X39" s="7" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="Y39" s="7" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>28</v>
@@ -4809,28 +4827,28 @@
         <v>29</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="G40" s="5">
         <v>2</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>335</v>
+        <v>395</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="J40" s="2">
         <v>2</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>335</v>
+        <v>395</v>
       </c>
       <c r="L40" s="3" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M40" s="3" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="N40" s="2">
         <v>3</v>
@@ -4842,42 +4860,42 @@
         <v>0</v>
       </c>
       <c r="Q40" s="3" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="R40" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S40" s="3" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="T40" s="3" t="s">
-        <v>391</v>
+        <v>158</v>
       </c>
       <c r="U40" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V40" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W40" s="3" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="X40" s="3" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="Y40" s="3" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="D41" s="8" t="s">
         <v>28</v>
@@ -4886,28 +4904,28 @@
         <v>29</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="G41" s="9">
         <v>3</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>202</v>
+        <v>144</v>
       </c>
       <c r="I41" s="7" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="J41" s="6">
         <v>3</v>
       </c>
       <c r="K41" s="7" t="s">
-        <v>202</v>
+        <v>144</v>
       </c>
       <c r="L41" s="7" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M41" s="7" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="N41" s="6">
         <v>5</v>
@@ -4919,31 +4937,31 @@
         <v>0</v>
       </c>
       <c r="Q41" s="7" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="R41" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S41" s="7" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="T41" s="7" t="s">
-        <v>310</v>
+        <v>70</v>
       </c>
       <c r="U41" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V41" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W41" s="7" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="X41" s="7" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="Y41" s="7" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-collected traffic data: 2026-09-03 10:15 AM IST [10_00 AM]
</commit_message>
<xml_diff>
--- a/output/excel/Kolkata_Traffic_Data_2026-09-03.xlsx
+++ b/output/excel/Kolkata_Traffic_Data_2026-09-03.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1664" uniqueCount="651">
   <si>
     <t>Route ID</t>
   </si>
@@ -1319,12 +1320,830 @@
   <si>
     <t>screenshots/2026-09-03/12_00 AM/S19_Bagha_Jatin___Baishnabghata/bus.jpg</t>
   </si>
+  <si>
+    <t>10_00 AM</t>
+  </si>
+  <si>
+    <t>Thursday (Weekday) - 10_00 AM</t>
+  </si>
+  <si>
+    <t>22.1 km</t>
+  </si>
+  <si>
+    <t>15.1</t>
+  </si>
+  <si>
+    <t>19.2</t>
+  </si>
+  <si>
+    <t>-19 min (Bike Faster)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 hr 9 min
+10:28 AM—11:37 AM
+AC-52</t>
+  </si>
+  <si>
+    <t>0.78x</t>
+  </si>
+  <si>
+    <t>0 Min Walk Time (Direct Boarding) + Direct Route (No Transfers)</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M01_DH_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M01_DH_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M01_DH_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>15.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 min
+10:02 AM—10:23 AM
+214</t>
+  </si>
+  <si>
+    <t>0.84x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M02_B_T_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M02_B_T_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M02_B_T_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>25.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43 min
+10:11 AM—10:54 AM
+Barrackpore Chiriamore - Salap More</t>
+  </si>
+  <si>
+    <t>1.48x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M03_B_T_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M03_B_T_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M03_B_T_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>13.8 km</t>
+  </si>
+  <si>
+    <t>21.2</t>
+  </si>
+  <si>
+    <t>-5 min (Bike Faster)</t>
+  </si>
+  <si>
+    <t>25.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32 min
+10:20 AM—10:52 AM
+L238
+10:20 AM from Muchi Bazar
+Details</t>
+  </si>
+  <si>
+    <t>0.73x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M04_VIP_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M04_VIP_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M04_VIP_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>21.9</t>
+  </si>
+  <si>
+    <t>-4 min (Bike Faster)</t>
+  </si>
+  <si>
+    <t>17.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38 min
+10:16 AM—10:54 AM
+DN-17</t>
+  </si>
+  <si>
+    <t>1.09x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M05_Jessore_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M05_Jessore_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M05_Jessore_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>15.2</t>
+  </si>
+  <si>
+    <t>16.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 min
+10:09 AM—10:26 AM
+DN-9/1</t>
+  </si>
+  <si>
+    <t>0.89x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M06_Airport_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M06_Airport_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M06_Airport_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>10.9</t>
+  </si>
+  <si>
+    <t>13.7</t>
+  </si>
+  <si>
+    <t>15.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32 min
+10:10 AM—10:42 AM
+3D</t>
+  </si>
+  <si>
+    <t>0.71x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M07_APC_Bose_Rd/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M07_APC_Bose_Rd/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M07_APC_Bose_Rd/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 min
+10:08 AM—10:30 AM
+  214A</t>
+  </si>
+  <si>
+    <t>1.00x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M08_Bidhan_Sarani/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M08_Bidhan_Sarani/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M08_Bidhan_Sarani/bus.jpg</t>
+  </si>
+  <si>
+    <t>15.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 min
+10:05 AM—10:22 AM
+S-10</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M09_Central_Avenue__C_R_Avenue_/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M09_Central_Avenue__C_R_Avenue_/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M09_Central_Avenue__C_R_Avenue_/bus.jpg</t>
+  </si>
+  <si>
+    <t>15.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 min
+10:03 AM—10:10 AM
+S-12N</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M10_S_N_Banerjee_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M10_S_N_Banerjee_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M10_S_N_Banerjee_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>14.0</t>
+  </si>
+  <si>
+    <t>14.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+10:13 AM—10:26 AM
+24</t>
+  </si>
+  <si>
+    <t>0.72x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M11_M_G_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M11_M_G_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M11_M_G_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>9.8</t>
+  </si>
+  <si>
+    <t>15.6</t>
+  </si>
+  <si>
+    <t>-6 min (Bike Faster)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 min
+10:07 AM—10:16 AM
+KB-17</t>
+  </si>
+  <si>
+    <t>0.56x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M12_C_I_T_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M12_C_I_T_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M12_C_I_T_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>11.4</t>
+  </si>
+  <si>
+    <t>13.4</t>
+  </si>
+  <si>
+    <t>-3 min (Bike Faster)</t>
+  </si>
+  <si>
+    <t>12.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 min
+10:19 AM—10:37 AM
+234  </t>
+  </si>
+  <si>
+    <t>0.90x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M13_Sarat_Bose_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M13_Sarat_Bose_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M13_Sarat_Bose_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>16.4 km</t>
+  </si>
+  <si>
+    <t>14.9</t>
+  </si>
+  <si>
+    <t>-8 min (Bike Faster)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 hr
+10:05 AM—11:05 AM
+222  S-112</t>
+  </si>
+  <si>
+    <t>0.91x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M14_S_P_Mukherjee_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M14_S_P_Mukherjee_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M14_S_P_Mukherjee_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>6.8 km</t>
+  </si>
+  <si>
+    <t>14.6</t>
+  </si>
+  <si>
+    <t>18.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34 min
+10:26 AM—11:00 AM
+103  13A</t>
+  </si>
+  <si>
+    <t>1.21x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M15_Hazra_Road___S_P_Mukherjee_Road_connector/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M15_Hazra_Road___S_P_Mukherjee_Road_connector/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M15_Hazra_Road___S_P_Mukherjee_Road_connector/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 min
+10:27 AM—10:37 AM
+M-14</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M16_Gariahat_Road___Rashbehari_Avenue/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M16_Gariahat_Road___Rashbehari_Avenue/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M16_Gariahat_Road___Rashbehari_Avenue/bus.jpg</t>
+  </si>
+  <si>
+    <t>11.2</t>
+  </si>
+  <si>
+    <t>18.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 min
+10:36 AM—10:45 AM
+SD76</t>
+  </si>
+  <si>
+    <t>0.60x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M18_Chetla_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M18_Chetla_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M18_Chetla_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>4.3 km</t>
+  </si>
+  <si>
+    <t>13.6</t>
+  </si>
+  <si>
+    <t>16.1</t>
+  </si>
+  <si>
+    <t>19.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+10:24 AM—10:37 AM
+SD5</t>
+  </si>
+  <si>
+    <t>0.68x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M19_Taratala_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M19_Taratala_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M19_Taratala_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>15.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 min
+10:31 AM—10:55 AM
+ST-6</t>
+  </si>
+  <si>
+    <t>0.92x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M20_Prince_Anwar_Shah_Rd/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M20_Prince_Anwar_Shah_Rd/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M20_Prince_Anwar_Shah_Rd/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 min
+10:19 AM—10:29 AM
+S-9</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M21_Karunamoyee_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M21_Karunamoyee_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M21_Karunamoyee_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>15.0</t>
+  </si>
+  <si>
+    <t>22.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 min
+10:08 AM—10:23 AM
+S-22
+10:08 AM from Karunamayee
+Details</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M22_Canal_South_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M22_Canal_South_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M22_Canal_South_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>14.5</t>
+  </si>
+  <si>
+    <t>18.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+10:10 AM—10:23 AM
+Berachampa - Karunamoyee</t>
+  </si>
+  <si>
+    <t>0.76x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M23_VIP_Road_connector/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M23_VIP_Road_connector/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/M23_VIP_Road_connector/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 min
+10:10 AM—10:14 AM
+Kamal Gazi Bypass - Dankuni Housing</t>
+  </si>
+  <si>
+    <t>0.67x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S01_Baishnabghata_Patuli/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S01_Baishnabghata_Patuli/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S01_Baishnabghata_Patuli/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 min
+10:06 AM—10:10 AM
+Bagbazar - Garia Station</t>
+  </si>
+  <si>
+    <t>1.33x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S02_Patuli___Highland_Park/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S02_Patuli___Highland_Park/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S02_Patuli___Highland_Park/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 min
+10:10 AM—10:13 AM
+Bagbazar - Garia Station</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S03_Highland_Park___Ajaynagar/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S03_Highland_Park___Ajaynagar/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S03_Highland_Park___Ajaynagar/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 min
+10:10 AM—10:16 AM
+S-21</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S04_Ajaynagar___Kalikapur/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S04_Ajaynagar___Kalikapur/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S04_Ajaynagar___Kalikapur/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 min
+10:02 AM—10:06 AM
+Barasat - Baruipur</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S05_Kalikapur___Ruby/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S05_Kalikapur___Ruby/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S05_Kalikapur___Ruby/bus.jpg</t>
+  </si>
+  <si>
+    <t>21.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 min
+10:27 AM—10:41 AM
+EB-16</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S06_Ruby___Science_City/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S06_Ruby___Science_City/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S06_Ruby___Science_City/bus.jpg</t>
+  </si>
+  <si>
+    <t>22.8</t>
+  </si>
+  <si>
+    <t>19.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 min
+10:41 AM—10:47 AM
+EB-16</t>
+  </si>
+  <si>
+    <t>1.20x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S07_Science_City___Chingrighata/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S07_Science_City___Chingrighata/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S07_Science_City___Chingrighata/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16 min
+10:02 AM—10:18 AM
+239</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S08_Chingrighata___Sealdah/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S08_Chingrighata___Sealdah/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S08_Chingrighata___Sealdah/bus.jpg</t>
+  </si>
+  <si>
+    <t>12.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 min
+10:08 AM—10:22 AM
+  39A/2</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S09_Sealdah___Park_Circus/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S09_Sealdah___Park_Circus/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S09_Sealdah___Park_Circus/bus.jpg</t>
+  </si>
+  <si>
+    <t>20.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19 min
+10:14 AM—10:33 AM
+Santragachhi Bus Terminus - Regent Bus Stand  K-4</t>
+  </si>
+  <si>
+    <t>1.73x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S10_Park_Circus___Science_City/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S10_Park_Circus___Science_City/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S10_Park_Circus___Science_City/bus.jpg</t>
+  </si>
+  <si>
+    <t>11.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 min
+10:01 AM—10:10 AM
+45A
+10:02 AM from Zeeshan
+ 1 min
+Details</t>
+  </si>
+  <si>
+    <t>0.64x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S11_Park_Circus___Gariahat/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S11_Park_Circus___Gariahat/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S11_Park_Circus___Gariahat/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+10:04 AM—10:17 AM
+SD76</t>
+  </si>
+  <si>
+    <t>0.93x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S12_Gariahat___Ruby/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S12_Gariahat___Ruby/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S12_Gariahat___Ruby/bus.jpg</t>
+  </si>
+  <si>
+    <t>20.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 min
+10:16 AM—10:23 AM
+13C</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S13_Gariahat___Mallick_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S13_Gariahat___Mallick_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S13_Gariahat___Mallick_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>19.1</t>
+  </si>
+  <si>
+    <t>16.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+10:26 AM—10:39 AM
+S-4D</t>
+  </si>
+  <si>
+    <t>1.18x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S14_Jadavpur_Police_St____Kalikapur/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S14_Jadavpur_Police_St____Kalikapur/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S14_Jadavpur_Police_St____Kalikapur/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 min
+10:08 AM—10:12 AM
+1A</t>
+  </si>
+  <si>
+    <t>0.80x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S15_Mallick_Road___Jadavpur_Sulekha/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S15_Mallick_Road___Jadavpur_Sulekha/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S15_Mallick_Road___Jadavpur_Sulekha/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 min
+10:02 AM—10:12 AM
+S-9</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S16_Jadavpur_Sulekha___Ajay_Nagar/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S16_Jadavpur_Sulekha___Ajay_Nagar/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S16_Jadavpur_Sulekha___Ajay_Nagar/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 min
+10:07 AM—10:10 AM
+45B
+10:07 AM from Sulekha More
+Details</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S17_Jadavpur_Sulekha___Bagha_Jatin/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S17_Jadavpur_Sulekha___Bagha_Jatin/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S17_Jadavpur_Sulekha___Bagha_Jatin/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 min
+10:30 AM—10:35 AM
+45B</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S19_Bagha_Jatin___Baishnabghata/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S19_Bagha_Jatin___Baishnabghata/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/10_00 AM/S19_Bagha_Jatin___Baishnabghata/bus.jpg</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1346,6 +2165,18 @@
     <font>
       <b/>
       <color rgb="006100"/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="9C6500"/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="9C0006"/>
       <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
@@ -1411,7 +2242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1438,6 +2269,12 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4969,4 +5806,3197 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Y41"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="33" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="25" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="29" customWidth="1"/>
+    <col min="16" max="16" width="30" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="18" max="18" width="21" customWidth="1"/>
+    <col min="19" max="19" width="45" customWidth="1"/>
+    <col min="20" max="20" width="20" customWidth="1"/>
+    <col min="21" max="21" width="23" customWidth="1"/>
+    <col min="22" max="25" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="G2" s="2">
+        <v>88</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="J2" s="2">
+        <v>69</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="N2" s="2">
+        <v>69</v>
+      </c>
+      <c r="O2" s="2">
+        <v>69</v>
+      </c>
+      <c r="P2" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="9">
+        <v>25</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3" s="6">
+        <v>23</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>420</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="N3" s="6">
+        <v>21</v>
+      </c>
+      <c r="O3" s="6">
+        <v>21</v>
+      </c>
+      <c r="P3" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S3" s="7" t="s">
+        <v>421</v>
+      </c>
+      <c r="T3" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="U3" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V3" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W3" s="7" t="s">
+        <v>423</v>
+      </c>
+      <c r="X3" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="Y3" s="7" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="5">
+        <v>29</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="2">
+        <v>27</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="N4" s="2">
+        <v>43</v>
+      </c>
+      <c r="O4" s="2">
+        <v>43</v>
+      </c>
+      <c r="P4" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W4" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="X4" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="Y4" s="3" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="G5" s="6">
+        <v>44</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="J5" s="6">
+        <v>39</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="N5" s="6">
+        <v>32</v>
+      </c>
+      <c r="O5" s="6">
+        <v>32</v>
+      </c>
+      <c r="P5" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="R5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S5" s="7" t="s">
+        <v>436</v>
+      </c>
+      <c r="T5" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="U5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V5" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W5" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="X5" s="7" t="s">
+        <v>439</v>
+      </c>
+      <c r="Y5" s="7" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G6" s="2">
+        <v>35</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="2">
+        <v>31</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="N6" s="2">
+        <v>38</v>
+      </c>
+      <c r="O6" s="2">
+        <v>38</v>
+      </c>
+      <c r="P6" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S6" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="U6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W6" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="X6" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G7" s="9">
+        <v>19</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="J7" s="6">
+        <v>17</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="N7" s="6">
+        <v>17</v>
+      </c>
+      <c r="O7" s="6">
+        <v>17</v>
+      </c>
+      <c r="P7" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S7" s="7" t="s">
+        <v>451</v>
+      </c>
+      <c r="T7" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="U7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V7" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W7" s="7" t="s">
+        <v>453</v>
+      </c>
+      <c r="X7" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="Y7" s="7" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G8" s="2">
+        <v>45</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="J8" s="2">
+        <v>36</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="N8" s="2">
+        <v>32</v>
+      </c>
+      <c r="O8" s="2">
+        <v>32</v>
+      </c>
+      <c r="P8" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S8" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="U8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V8" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W8" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="X8" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="Y8" s="3" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" s="9">
+        <v>22</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J9" s="6">
+        <v>21</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="N9" s="6">
+        <v>22</v>
+      </c>
+      <c r="O9" s="6">
+        <v>22</v>
+      </c>
+      <c r="P9" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S9" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="T9" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="U9" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V9" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W9" s="7" t="s">
+        <v>466</v>
+      </c>
+      <c r="X9" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="Y9" s="7" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G10" s="5">
+        <v>19</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="J10" s="2">
+        <v>17</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="N10" s="2">
+        <v>17</v>
+      </c>
+      <c r="O10" s="2">
+        <v>17</v>
+      </c>
+      <c r="P10" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="R10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S10" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="T10" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="U10" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V10" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W10" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="X10" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="Y10" s="3" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G11" s="6">
+        <v>9</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="J11" s="6">
+        <v>8</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="N11" s="6">
+        <v>7</v>
+      </c>
+      <c r="O11" s="6">
+        <v>7</v>
+      </c>
+      <c r="P11" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S11" s="7" t="s">
+        <v>475</v>
+      </c>
+      <c r="T11" s="7" t="s">
+        <v>415</v>
+      </c>
+      <c r="U11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V11" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W11" s="7" t="s">
+        <v>476</v>
+      </c>
+      <c r="X11" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="Y11" s="7" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="G12" s="5">
+        <v>18</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="J12" s="2">
+        <v>17</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="N12" s="2">
+        <v>13</v>
+      </c>
+      <c r="O12" s="2">
+        <v>13</v>
+      </c>
+      <c r="P12" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="R12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S12" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="T12" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="U12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V12" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W12" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="X12" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="Y12" s="3" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="G13" s="9">
+        <v>16</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="J13" s="6">
+        <v>10</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="N13" s="6">
+        <v>9</v>
+      </c>
+      <c r="O13" s="6">
+        <v>9</v>
+      </c>
+      <c r="P13" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S13" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="T13" s="7" t="s">
+        <v>490</v>
+      </c>
+      <c r="U13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V13" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W13" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="X13" s="7" t="s">
+        <v>492</v>
+      </c>
+      <c r="Y13" s="7" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G14" s="2">
+        <v>20</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="J14" s="2">
+        <v>17</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="N14" s="2">
+        <v>18</v>
+      </c>
+      <c r="O14" s="2">
+        <v>18</v>
+      </c>
+      <c r="P14" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="R14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S14" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="T14" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="U14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V14" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W14" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="X14" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="Y14" s="3" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="G15" s="6">
+        <v>66</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>504</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="J15" s="6">
+        <v>58</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="N15" s="6">
+        <v>60</v>
+      </c>
+      <c r="O15" s="6">
+        <v>60</v>
+      </c>
+      <c r="P15" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S15" s="7" t="s">
+        <v>506</v>
+      </c>
+      <c r="T15" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V15" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W15" s="7" t="s">
+        <v>508</v>
+      </c>
+      <c r="X15" s="7" t="s">
+        <v>509</v>
+      </c>
+      <c r="Y15" s="7" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="G16" s="2">
+        <v>28</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="J16" s="2">
+        <v>22</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="N16" s="2">
+        <v>34</v>
+      </c>
+      <c r="O16" s="2">
+        <v>34</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="R16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S16" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="T16" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="U16" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W16" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="X16" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="Y16" s="3" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="G17" s="9">
+        <v>11</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>469</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J17" s="6">
+        <v>10</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="N17" s="6">
+        <v>10</v>
+      </c>
+      <c r="O17" s="6">
+        <v>10</v>
+      </c>
+      <c r="P17" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="R17" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S17" s="7" t="s">
+        <v>519</v>
+      </c>
+      <c r="T17" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="U17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V17" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W17" s="7" t="s">
+        <v>520</v>
+      </c>
+      <c r="X17" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="Y17" s="7" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="G18" s="2">
+        <v>15</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="J18" s="2">
+        <v>12</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="N18" s="2">
+        <v>9</v>
+      </c>
+      <c r="O18" s="2">
+        <v>9</v>
+      </c>
+      <c r="P18" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="3" t="s">
+        <v>524</v>
+      </c>
+      <c r="R18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S18" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="T18" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="U18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V18" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W18" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="X18" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="Y18" s="3" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="G19" s="6">
+        <v>19</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="J19" s="6">
+        <v>16</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="N19" s="6">
+        <v>13</v>
+      </c>
+      <c r="O19" s="6">
+        <v>13</v>
+      </c>
+      <c r="P19" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="R19" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S19" s="7" t="s">
+        <v>534</v>
+      </c>
+      <c r="T19" s="7" t="s">
+        <v>535</v>
+      </c>
+      <c r="U19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V19" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W19" s="7" t="s">
+        <v>536</v>
+      </c>
+      <c r="X19" s="7" t="s">
+        <v>537</v>
+      </c>
+      <c r="Y19" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="G20" s="5">
+        <v>26</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>539</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="J20" s="2">
+        <v>23</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="N20" s="2">
+        <v>24</v>
+      </c>
+      <c r="O20" s="2">
+        <v>24</v>
+      </c>
+      <c r="P20" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="R20" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S20" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="T20" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="U20" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V20" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W20" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="X20" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="Y20" s="3" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="G21" s="9">
+        <v>11</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="J21" s="6">
+        <v>10</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="N21" s="6">
+        <v>10</v>
+      </c>
+      <c r="O21" s="6">
+        <v>10</v>
+      </c>
+      <c r="P21" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="R21" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S21" s="7" t="s">
+        <v>545</v>
+      </c>
+      <c r="T21" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="U21" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V21" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W21" s="7" t="s">
+        <v>546</v>
+      </c>
+      <c r="X21" s="7" t="s">
+        <v>547</v>
+      </c>
+      <c r="Y21" s="7" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="G22" s="2">
+        <v>22</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="J22" s="2">
+        <v>19</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="M22" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="N22" s="2">
+        <v>15</v>
+      </c>
+      <c r="O22" s="2">
+        <v>15</v>
+      </c>
+      <c r="P22" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="R22" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S22" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="T22" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="U22" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V22" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W22" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="X22" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="Y22" s="3" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="G23" s="6">
+        <v>17</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>555</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="J23" s="6">
+        <v>16</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="N23" s="6">
+        <v>13</v>
+      </c>
+      <c r="O23" s="6">
+        <v>13</v>
+      </c>
+      <c r="P23" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="7" t="s">
+        <v>556</v>
+      </c>
+      <c r="R23" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S23" s="7" t="s">
+        <v>557</v>
+      </c>
+      <c r="T23" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V23" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W23" s="7" t="s">
+        <v>559</v>
+      </c>
+      <c r="X23" s="7" t="s">
+        <v>560</v>
+      </c>
+      <c r="Y23" s="7" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="G24" s="5">
+        <v>6</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="J24" s="2">
+        <v>5</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="N24" s="2">
+        <v>4</v>
+      </c>
+      <c r="O24" s="2">
+        <v>4</v>
+      </c>
+      <c r="P24" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="R24" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S24" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="T24" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="U24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V24" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W24" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="X24" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="Y24" s="3" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="G25" s="9">
+        <v>3</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="J25" s="6">
+        <v>3</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="N25" s="6">
+        <v>4</v>
+      </c>
+      <c r="O25" s="6">
+        <v>4</v>
+      </c>
+      <c r="P25" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="R25" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S25" s="7" t="s">
+        <v>567</v>
+      </c>
+      <c r="T25" s="7" t="s">
+        <v>568</v>
+      </c>
+      <c r="U25" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V25" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W25" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="X25" s="7" t="s">
+        <v>570</v>
+      </c>
+      <c r="Y25" s="7" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="G26" s="5">
+        <v>2</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="J26" s="2">
+        <v>2</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="N26" s="2">
+        <v>3</v>
+      </c>
+      <c r="O26" s="2">
+        <v>3</v>
+      </c>
+      <c r="P26" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="R26" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S26" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="T26" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="U26" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V26" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W26" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="X26" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="Y26" s="3" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="G27" s="9">
+        <v>4</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="J27" s="6">
+        <v>4</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="M27" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="N27" s="6">
+        <v>6</v>
+      </c>
+      <c r="O27" s="6">
+        <v>6</v>
+      </c>
+      <c r="P27" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="R27" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S27" s="7" t="s">
+        <v>576</v>
+      </c>
+      <c r="T27" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="U27" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V27" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W27" s="7" t="s">
+        <v>577</v>
+      </c>
+      <c r="X27" s="7" t="s">
+        <v>578</v>
+      </c>
+      <c r="Y27" s="7" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="G28" s="10">
+        <v>6</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="J28" s="2">
+        <v>4</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M28" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="N28" s="2">
+        <v>4</v>
+      </c>
+      <c r="O28" s="2">
+        <v>4</v>
+      </c>
+      <c r="P28" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="R28" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S28" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="T28" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="U28" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V28" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W28" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="X28" s="3" t="s">
+        <v>582</v>
+      </c>
+      <c r="Y28" s="3" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="G29" s="6">
+        <v>13</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>513</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="J29" s="6">
+        <v>11</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>584</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M29" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="N29" s="6">
+        <v>14</v>
+      </c>
+      <c r="O29" s="6">
+        <v>14</v>
+      </c>
+      <c r="P29" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="R29" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S29" s="7" t="s">
+        <v>585</v>
+      </c>
+      <c r="T29" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="U29" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V29" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W29" s="7" t="s">
+        <v>586</v>
+      </c>
+      <c r="X29" s="7" t="s">
+        <v>587</v>
+      </c>
+      <c r="Y29" s="7" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="G30" s="5">
+        <v>5</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>589</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="J30" s="2">
+        <v>5</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>589</v>
+      </c>
+      <c r="L30" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M30" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="N30" s="2">
+        <v>6</v>
+      </c>
+      <c r="O30" s="2">
+        <v>6</v>
+      </c>
+      <c r="P30" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="R30" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S30" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="T30" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="U30" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V30" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W30" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="X30" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="Y30" s="3" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="G31" s="9">
+        <v>18</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="J31" s="6">
+        <v>16</v>
+      </c>
+      <c r="K31" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M31" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="N31" s="6">
+        <v>16</v>
+      </c>
+      <c r="O31" s="6">
+        <v>16</v>
+      </c>
+      <c r="P31" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="R31" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S31" s="7" t="s">
+        <v>596</v>
+      </c>
+      <c r="T31" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="U31" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V31" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W31" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="X31" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="Y31" s="7" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G32" s="5">
+        <v>12</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="J32" s="2">
+        <v>11</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="L32" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="N32" s="2">
+        <v>14</v>
+      </c>
+      <c r="O32" s="2">
+        <v>14</v>
+      </c>
+      <c r="P32" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="R32" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S32" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="T32" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="U32" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V32" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W32" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="X32" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="Y32" s="3" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="G33" s="6">
+        <v>11</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="J33" s="6">
+        <v>10</v>
+      </c>
+      <c r="K33" s="7" t="s">
+        <v>589</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="N33" s="6">
+        <v>19</v>
+      </c>
+      <c r="O33" s="6">
+        <v>19</v>
+      </c>
+      <c r="P33" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="R33" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S33" s="7" t="s">
+        <v>606</v>
+      </c>
+      <c r="T33" s="7" t="s">
+        <v>607</v>
+      </c>
+      <c r="U33" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V33" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W33" s="7" t="s">
+        <v>608</v>
+      </c>
+      <c r="X33" s="7" t="s">
+        <v>609</v>
+      </c>
+      <c r="Y33" s="7" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="G34" s="2">
+        <v>14</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="J34" s="2">
+        <v>12</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M34" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="N34" s="2">
+        <v>9</v>
+      </c>
+      <c r="O34" s="2">
+        <v>9</v>
+      </c>
+      <c r="P34" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="R34" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="S34" s="3" t="s">
+        <v>612</v>
+      </c>
+      <c r="T34" s="3" t="s">
+        <v>613</v>
+      </c>
+      <c r="U34" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V34" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W34" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="X34" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="Y34" s="3" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="G35" s="11">
+        <v>14</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="J35" s="6">
+        <v>13</v>
+      </c>
+      <c r="K35" s="7" t="s">
+        <v>556</v>
+      </c>
+      <c r="L35" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M35" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="N35" s="6">
+        <v>13</v>
+      </c>
+      <c r="O35" s="6">
+        <v>13</v>
+      </c>
+      <c r="P35" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="7" t="s">
+        <v>556</v>
+      </c>
+      <c r="R35" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S35" s="7" t="s">
+        <v>617</v>
+      </c>
+      <c r="T35" s="7" t="s">
+        <v>618</v>
+      </c>
+      <c r="U35" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V35" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W35" s="7" t="s">
+        <v>619</v>
+      </c>
+      <c r="X35" s="7" t="s">
+        <v>620</v>
+      </c>
+      <c r="Y35" s="7" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="G36" s="5">
+        <v>7</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="J36" s="2">
+        <v>6</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="N36" s="2">
+        <v>7</v>
+      </c>
+      <c r="O36" s="2">
+        <v>7</v>
+      </c>
+      <c r="P36" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R36" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S36" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="T36" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="U36" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V36" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W36" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="X36" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="Y36" s="3" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="G37" s="9">
+        <v>11</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="J37" s="6">
+        <v>10</v>
+      </c>
+      <c r="K37" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="L37" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M37" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="N37" s="6">
+        <v>13</v>
+      </c>
+      <c r="O37" s="6">
+        <v>13</v>
+      </c>
+      <c r="P37" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="7" t="s">
+        <v>628</v>
+      </c>
+      <c r="R37" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S37" s="7" t="s">
+        <v>629</v>
+      </c>
+      <c r="T37" s="7" t="s">
+        <v>630</v>
+      </c>
+      <c r="U37" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V37" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W37" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="X37" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="Y37" s="7" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="G38" s="5">
+        <v>5</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="J38" s="2">
+        <v>4</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M38" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="N38" s="2">
+        <v>4</v>
+      </c>
+      <c r="O38" s="2">
+        <v>4</v>
+      </c>
+      <c r="P38" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="R38" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S38" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="T38" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="U38" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V38" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W38" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="X38" s="3" t="s">
+        <v>637</v>
+      </c>
+      <c r="Y38" s="3" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="G39" s="9">
+        <v>10</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="J39" s="6">
+        <v>9</v>
+      </c>
+      <c r="K39" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="L39" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M39" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="N39" s="6">
+        <v>10</v>
+      </c>
+      <c r="O39" s="6">
+        <v>10</v>
+      </c>
+      <c r="P39" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="R39" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S39" s="7" t="s">
+        <v>639</v>
+      </c>
+      <c r="T39" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="U39" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V39" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W39" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="X39" s="7" t="s">
+        <v>641</v>
+      </c>
+      <c r="Y39" s="7" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="G40" s="5">
+        <v>3</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="J40" s="2">
+        <v>3</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="L40" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M40" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="N40" s="2">
+        <v>3</v>
+      </c>
+      <c r="O40" s="2">
+        <v>3</v>
+      </c>
+      <c r="P40" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="R40" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S40" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="T40" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="U40" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V40" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W40" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="X40" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="Y40" s="3" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="G41" s="6">
+        <v>5</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="J41" s="6">
+        <v>5</v>
+      </c>
+      <c r="K41" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="L41" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="M41" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="N41" s="6">
+        <v>5</v>
+      </c>
+      <c r="O41" s="6">
+        <v>5</v>
+      </c>
+      <c r="P41" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="R41" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S41" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="T41" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="U41" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V41" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W41" s="7" t="s">
+        <v>648</v>
+      </c>
+      <c r="X41" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y41" s="7" t="s">
+        <v>650</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Y1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Auto-collected traffic data: 2026-09-03 01:15 PM IST [01_00 PM]
</commit_message>
<xml_diff>
--- a/output/excel/Kolkata_Traffic_Data_2026-09-03.xlsx
+++ b/output/excel/Kolkata_Traffic_Data_2026-09-03.xlsx
@@ -6,13 +6,14 @@
   <sheets>
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="01_00 PM" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1664" uniqueCount="651">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2501" uniqueCount="864">
   <si>
     <t>Route ID</t>
   </si>
@@ -2137,6 +2138,720 @@
   </si>
   <si>
     <t>screenshots/2026-09-03/10_00 AM/S19_Bagha_Jatin___Baishnabghata/bus.jpg</t>
+  </si>
+  <si>
+    <t>01_00 PM</t>
+  </si>
+  <si>
+    <t>Thursday (Weekday) - 01_00 PM</t>
+  </si>
+  <si>
+    <t>16.0</t>
+  </si>
+  <si>
+    <t>-11 min (Bike Faster)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 hr 9 min
+7:28 AM—8:37 AM
+AC-52</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M01_DH_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M01_DH_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M01_DH_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>12.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 min
+1:48 AM—2:09 AM
+78
+1:48 AM from Shyambazar
+Details</t>
+  </si>
+  <si>
+    <t>0.75x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M02_B_T_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M02_B_T_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M02_B_T_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43 min
+5:09 AM—5:52 AM
+78</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M03_B_T_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M03_B_T_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M03_B_T_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>16.6</t>
+  </si>
+  <si>
+    <t>-10 min (Bike Faster)</t>
+  </si>
+  <si>
+    <t>20.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">41 min
+1:53 AM—2:34 AM
+91C  </t>
+  </si>
+  <si>
+    <t>0.82x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M04_VIP_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M04_VIP_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M04_VIP_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>18.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42 min
+4:27 AM—5:09 AM
+DN-18  </t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M05_Jessore_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M05_Jessore_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M05_Jessore_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>7.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">41 min
+3:14 AM—3:55 AM
+93  </t>
+  </si>
+  <si>
+    <t>2.05x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M06_Airport_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M06_Airport_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M06_Airport_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>11.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29 min
+2:13 AM—2:42 AM
+227
+2:13 AM from Shyambazar 5 Point
+Details</t>
+  </si>
+  <si>
+    <t>0.62x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M07_APC_Bose_Rd/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M07_APC_Bose_Rd/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M07_APC_Bose_Rd/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 min
+2:58 AM—3:20 AM
+34B</t>
+  </si>
+  <si>
+    <t>0.79x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M08_Bidhan_Sarani/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M08_Bidhan_Sarani/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M08_Bidhan_Sarani/bus.jpg</t>
+  </si>
+  <si>
+    <t>14.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 min
+2:56 AM—3:20 AM
+  34B</t>
+  </si>
+  <si>
+    <t>0.96x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M09_Central_Avenue__C_R_Avenue_/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M09_Central_Avenue__C_R_Avenue_/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M09_Central_Avenue__C_R_Avenue_/bus.jpg</t>
+  </si>
+  <si>
+    <t>10.6</t>
+  </si>
+  <si>
+    <t>13.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 min
+1:53 AM—2:00 AM
+S-12N</t>
+  </si>
+  <si>
+    <t>0.54x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M10_S_N_Banerjee_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M10_S_N_Banerjee_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M10_S_N_Banerjee_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+3:33 AM—3:46 AM
+28</t>
+  </si>
+  <si>
+    <t>0.50x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M11_M_G_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M11_M_G_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M11_M_G_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>14.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 min
+2:16 AM—2:25 AM
+45</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M12_C_I_T_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M12_C_I_T_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M12_C_I_T_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+2:43 AM—2:56 AM
+221</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M13_Sarat_Bose_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M13_Sarat_Bose_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M13_Sarat_Bose_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>16.6 km</t>
+  </si>
+  <si>
+    <t>21.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">46 min
+3:46 AM—4:32 AM
+239    34712  </t>
+  </si>
+  <si>
+    <t>0.70x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M14_S_P_Mukherjee_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M14_S_P_Mukherjee_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M14_S_P_Mukherjee_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>4.9 km</t>
+  </si>
+  <si>
+    <t>8.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33 min
+4:58 AM—5:31 AM
+  S-131</t>
+  </si>
+  <si>
+    <t>1.22x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M15_Hazra_Road___S_P_Mukherjee_Road_connector/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M15_Hazra_Road___S_P_Mukherjee_Road_connector/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M15_Hazra_Road___S_P_Mukherjee_Road_connector/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 min
+2:22 AM—2:43 AM
+1  </t>
+  </si>
+  <si>
+    <t>1.40x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M16_Gariahat_Road___Rashbehari_Avenue/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M16_Gariahat_Road___Rashbehari_Avenue/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M16_Gariahat_Road___Rashbehari_Avenue/bus.jpg</t>
+  </si>
+  <si>
+    <t>3.0 km</t>
+  </si>
+  <si>
+    <t>10.0</t>
+  </si>
+  <si>
+    <t>8.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 min
+2:19 AM—2:40 AM
+  12C/1</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M18_Chetla_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M18_Chetla_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M18_Chetla_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>8.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47 min
+3:39 AM—4:26 AM
+  34112  </t>
+  </si>
+  <si>
+    <t>1.68x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M19_Taratala_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M19_Taratala_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M19_Taratala_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>7.4 km</t>
+  </si>
+  <si>
+    <t>19.3</t>
+  </si>
+  <si>
+    <t>5.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 hr 20 min
+2:05 AM—3:25 AM
+  1B  </t>
+  </si>
+  <si>
+    <t>3.08x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M20_Prince_Anwar_Shah_Rd/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M20_Prince_Anwar_Shah_Rd/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M20_Prince_Anwar_Shah_Rd/bus.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M21_Karunamoyee_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M21_Karunamoyee_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M21_Karunamoyee_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>20.6</t>
+  </si>
+  <si>
+    <t>8.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39 min
+1:01 AM—1:40 AM
+  S-12N  
+1:30 AM from Nabadiganta Bhavan
+ 33 min
+Details</t>
+  </si>
+  <si>
+    <t>2.17x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M22_Canal_South_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M22_Canal_South_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M22_Canal_South_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>9.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 min
+3:42 AM—4:08 AM
+  215A  </t>
+  </si>
+  <si>
+    <t>1.63x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M23_VIP_Road_connector/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M23_VIP_Road_connector/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/M23_VIP_Road_connector/bus.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S01_Baishnabghata_Patuli/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S01_Baishnabghata_Patuli/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S01_Baishnabghata_Patuli/bus.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S02_Patuli___Highland_Park/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S02_Patuli___Highland_Park/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S02_Patuli___Highland_Park/bus.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S03_Highland_Park___Ajaynagar/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S03_Highland_Park___Ajaynagar/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S03_Highland_Park___Ajaynagar/bus.jpg</t>
+  </si>
+  <si>
+    <t>9.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 min
+1:54 AM—2:05 AM
+  1</t>
+  </si>
+  <si>
+    <t>2.75x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S04_Ajaynagar___Kalikapur/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S04_Ajaynagar___Kalikapur/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S04_Ajaynagar___Kalikapur/bus.jpg</t>
+  </si>
+  <si>
+    <t>24.0</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S05_Kalikapur___Ruby/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S05_Kalikapur___Ruby/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S05_Kalikapur___Ruby/bus.jpg</t>
+  </si>
+  <si>
+    <t>26.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 min
+5:14 AM—5:40 AM
+24A/1  </t>
+  </si>
+  <si>
+    <t>2.89x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S06_Ruby___Science_City/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S06_Ruby___Science_City/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S06_Ruby___Science_City/bus.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S07_Science_City___Chingrighata/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S07_Science_City___Chingrighata/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S07_Science_City___Chingrighata/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 min
+1:37 AM—1:52 AM
+S-12N</t>
+  </si>
+  <si>
+    <t>0.83x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S08_Chingrighata___Sealdah/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S08_Chingrighata___Sealdah/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S08_Chingrighata___Sealdah/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45 min
+1:17 AM—2:02 AM
+S-12N  230  </t>
+  </si>
+  <si>
+    <t>3.46x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S09_Sealdah___Park_Circus/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S09_Sealdah___Park_Circus/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S09_Sealdah___Park_Circus/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19 min
+5:55 AM—6:14 AM
+Ecospace Amity University - Andul Station Road  </t>
+  </si>
+  <si>
+    <t>3.17x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S10_Park_Circus___Science_City/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S10_Park_Circus___Science_City/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S10_Park_Circus___Science_City/bus.jpg</t>
+  </si>
+  <si>
+    <t>14.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 min
+2:25 AM—2:37 AM
+45</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S11_Park_Circus___Gariahat/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S11_Park_Circus___Gariahat/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S11_Park_Circus___Gariahat/bus.jpg</t>
+  </si>
+  <si>
+    <t>20.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 min
+3:43 AM—3:57 AM
+18B/1</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S12_Gariahat___Ruby/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S12_Gariahat___Ruby/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S12_Gariahat___Ruby/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 min
+2:35 AM—2:42 AM
+45</t>
+  </si>
+  <si>
+    <t>0.88x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S13_Gariahat___Mallick_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S13_Gariahat___Mallick_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S13_Gariahat___Mallick_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>23.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42 min
+2:43 AM—3:25 AM
+1B  </t>
+  </si>
+  <si>
+    <t>4.20x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S14_Jadavpur_Police_St____Kalikapur/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S14_Jadavpur_Police_St____Kalikapur/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S14_Jadavpur_Police_St____Kalikapur/bus.jpg</t>
+  </si>
+  <si>
+    <t>11.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 min
+1:38 AM—1:45 AM
+45</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S15_Mallick_Road___Jadavpur_Sulekha/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S15_Mallick_Road___Jadavpur_Sulekha/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S15_Mallick_Road___Jadavpur_Sulekha/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 min
+2:50 AM—3:01 AM
+1B</t>
+  </si>
+  <si>
+    <t>1.10x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S16_Jadavpur_Sulekha___Ajay_Nagar/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S16_Jadavpur_Sulekha___Ajay_Nagar/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S16_Jadavpur_Sulekha___Ajay_Nagar/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 min
+5:58 AM—6:01 AM
+13C</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S17_Jadavpur_Sulekha___Bagha_Jatin/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S17_Jadavpur_Sulekha___Bagha_Jatin/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S17_Jadavpur_Sulekha___Bagha_Jatin/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 min
+1:46 AM—1:51 AM
+45</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S19_Bagha_Jatin___Baishnabghata/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S19_Bagha_Jatin___Baishnabghata/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/01_00 PM/S19_Bagha_Jatin___Baishnabghata/bus.jpg</t>
   </si>
 </sst>
 </file>
@@ -8997,6 +9712,3199 @@
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Y41"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="33" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="25" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="29" customWidth="1"/>
+    <col min="16" max="16" width="30" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="18" max="18" width="21" customWidth="1"/>
+    <col min="19" max="19" width="45" customWidth="1"/>
+    <col min="20" max="20" width="20" customWidth="1"/>
+    <col min="21" max="21" width="23" customWidth="1"/>
+    <col min="22" max="25" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="2">
+        <v>74</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J2" s="2">
+        <v>63</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N2" s="2">
+        <v>69</v>
+      </c>
+      <c r="O2" s="2">
+        <v>69</v>
+      </c>
+      <c r="P2" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>618</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>656</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>657</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="9">
+        <v>28</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>659</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3" s="6">
+        <v>23</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>420</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="N3" s="6">
+        <v>21</v>
+      </c>
+      <c r="O3" s="6">
+        <v>21</v>
+      </c>
+      <c r="P3" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S3" s="7" t="s">
+        <v>660</v>
+      </c>
+      <c r="T3" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="U3" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V3" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W3" s="7" t="s">
+        <v>662</v>
+      </c>
+      <c r="X3" s="7" t="s">
+        <v>663</v>
+      </c>
+      <c r="Y3" s="7" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="2">
+        <v>29</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="2">
+        <v>27</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="N4" s="2">
+        <v>43</v>
+      </c>
+      <c r="O4" s="2">
+        <v>43</v>
+      </c>
+      <c r="P4" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>665</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W4" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="X4" s="3" t="s">
+        <v>667</v>
+      </c>
+      <c r="Y4" s="3" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="G5" s="6">
+        <v>50</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>669</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="J5" s="6">
+        <v>40</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="N5" s="6">
+        <v>41</v>
+      </c>
+      <c r="O5" s="6">
+        <v>41</v>
+      </c>
+      <c r="P5" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>671</v>
+      </c>
+      <c r="R5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S5" s="7" t="s">
+        <v>672</v>
+      </c>
+      <c r="T5" s="7" t="s">
+        <v>673</v>
+      </c>
+      <c r="U5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V5" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W5" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="X5" s="7" t="s">
+        <v>675</v>
+      </c>
+      <c r="Y5" s="7" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G6" s="2">
+        <v>45</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="2">
+        <v>37</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>677</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="N6" s="2">
+        <v>42</v>
+      </c>
+      <c r="O6" s="2">
+        <v>42</v>
+      </c>
+      <c r="P6" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S6" s="3" t="s">
+        <v>678</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>618</v>
+      </c>
+      <c r="U6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V6" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W6" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="X6" s="3" t="s">
+        <v>680</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G7" s="6">
+        <v>20</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="J7" s="6">
+        <v>17</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="N7" s="6">
+        <v>41</v>
+      </c>
+      <c r="O7" s="6">
+        <v>41</v>
+      </c>
+      <c r="P7" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S7" s="7" t="s">
+        <v>683</v>
+      </c>
+      <c r="T7" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="U7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V7" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W7" s="7" t="s">
+        <v>685</v>
+      </c>
+      <c r="X7" s="7" t="s">
+        <v>686</v>
+      </c>
+      <c r="Y7" s="7" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G8" s="5">
+        <v>47</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="J8" s="2">
+        <v>42</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="N8" s="2">
+        <v>29</v>
+      </c>
+      <c r="O8" s="2">
+        <v>29</v>
+      </c>
+      <c r="P8" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S8" s="3" t="s">
+        <v>689</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="U8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V8" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W8" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="X8" s="3" t="s">
+        <v>692</v>
+      </c>
+      <c r="Y8" s="3" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" s="9">
+        <v>28</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>659</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J9" s="6">
+        <v>24</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>549</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="N9" s="6">
+        <v>22</v>
+      </c>
+      <c r="O9" s="6">
+        <v>22</v>
+      </c>
+      <c r="P9" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S9" s="7" t="s">
+        <v>694</v>
+      </c>
+      <c r="T9" s="7" t="s">
+        <v>695</v>
+      </c>
+      <c r="U9" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V9" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W9" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="X9" s="7" t="s">
+        <v>697</v>
+      </c>
+      <c r="Y9" s="7" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G10" s="5">
+        <v>25</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="J10" s="2">
+        <v>21</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="N10" s="2">
+        <v>24</v>
+      </c>
+      <c r="O10" s="2">
+        <v>24</v>
+      </c>
+      <c r="P10" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="R10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S10" s="3" t="s">
+        <v>700</v>
+      </c>
+      <c r="T10" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="U10" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V10" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W10" s="3" t="s">
+        <v>702</v>
+      </c>
+      <c r="X10" s="3" t="s">
+        <v>703</v>
+      </c>
+      <c r="Y10" s="3" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G11" s="6">
+        <v>13</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>705</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="J11" s="6">
+        <v>10</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="N11" s="6">
+        <v>7</v>
+      </c>
+      <c r="O11" s="6">
+        <v>7</v>
+      </c>
+      <c r="P11" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S11" s="7" t="s">
+        <v>707</v>
+      </c>
+      <c r="T11" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="U11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V11" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W11" s="7" t="s">
+        <v>709</v>
+      </c>
+      <c r="X11" s="7" t="s">
+        <v>710</v>
+      </c>
+      <c r="Y11" s="7" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="G12" s="2">
+        <v>26</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="J12" s="2">
+        <v>20</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>706</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="N12" s="2">
+        <v>13</v>
+      </c>
+      <c r="O12" s="2">
+        <v>13</v>
+      </c>
+      <c r="P12" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="R12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S12" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="T12" s="3" t="s">
+        <v>713</v>
+      </c>
+      <c r="U12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V12" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W12" s="3" t="s">
+        <v>714</v>
+      </c>
+      <c r="X12" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="Y12" s="3" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="G13" s="9">
+        <v>11</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>717</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="J13" s="6">
+        <v>10</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="N13" s="6">
+        <v>9</v>
+      </c>
+      <c r="O13" s="6">
+        <v>9</v>
+      </c>
+      <c r="P13" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S13" s="7" t="s">
+        <v>718</v>
+      </c>
+      <c r="T13" s="7" t="s">
+        <v>673</v>
+      </c>
+      <c r="U13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V13" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W13" s="7" t="s">
+        <v>719</v>
+      </c>
+      <c r="X13" s="7" t="s">
+        <v>720</v>
+      </c>
+      <c r="Y13" s="7" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G14" s="5">
+        <v>21</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="J14" s="2">
+        <v>18</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="N14" s="2">
+        <v>13</v>
+      </c>
+      <c r="O14" s="2">
+        <v>13</v>
+      </c>
+      <c r="P14" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="R14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S14" s="3" t="s">
+        <v>722</v>
+      </c>
+      <c r="T14" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="U14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V14" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W14" s="3" t="s">
+        <v>723</v>
+      </c>
+      <c r="X14" s="3" t="s">
+        <v>724</v>
+      </c>
+      <c r="Y14" s="3" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>726</v>
+      </c>
+      <c r="G15" s="6">
+        <v>66</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>726</v>
+      </c>
+      <c r="J15" s="6">
+        <v>58</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>726</v>
+      </c>
+      <c r="N15" s="6">
+        <v>46</v>
+      </c>
+      <c r="O15" s="6">
+        <v>46</v>
+      </c>
+      <c r="P15" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>727</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S15" s="7" t="s">
+        <v>728</v>
+      </c>
+      <c r="T15" s="7" t="s">
+        <v>729</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V15" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W15" s="7" t="s">
+        <v>730</v>
+      </c>
+      <c r="X15" s="7" t="s">
+        <v>731</v>
+      </c>
+      <c r="Y15" s="7" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>733</v>
+      </c>
+      <c r="G16" s="2">
+        <v>27</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>733</v>
+      </c>
+      <c r="J16" s="2">
+        <v>22</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>733</v>
+      </c>
+      <c r="N16" s="2">
+        <v>33</v>
+      </c>
+      <c r="O16" s="2">
+        <v>33</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="3" t="s">
+        <v>734</v>
+      </c>
+      <c r="R16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S16" s="3" t="s">
+        <v>735</v>
+      </c>
+      <c r="T16" s="3" t="s">
+        <v>736</v>
+      </c>
+      <c r="U16" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W16" s="3" t="s">
+        <v>737</v>
+      </c>
+      <c r="X16" s="3" t="s">
+        <v>738</v>
+      </c>
+      <c r="Y16" s="3" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="G17" s="9">
+        <v>15</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>611</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J17" s="6">
+        <v>13</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>495</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="N17" s="6">
+        <v>21</v>
+      </c>
+      <c r="O17" s="6">
+        <v>21</v>
+      </c>
+      <c r="P17" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="R17" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S17" s="7" t="s">
+        <v>740</v>
+      </c>
+      <c r="T17" s="7" t="s">
+        <v>741</v>
+      </c>
+      <c r="U17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V17" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W17" s="7" t="s">
+        <v>742</v>
+      </c>
+      <c r="X17" s="7" t="s">
+        <v>743</v>
+      </c>
+      <c r="Y17" s="7" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>745</v>
+      </c>
+      <c r="G18" s="2">
+        <v>18</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>746</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>745</v>
+      </c>
+      <c r="J18" s="2">
+        <v>14</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>659</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>745</v>
+      </c>
+      <c r="N18" s="2">
+        <v>21</v>
+      </c>
+      <c r="O18" s="2">
+        <v>21</v>
+      </c>
+      <c r="P18" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="R18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S18" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="T18" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="U18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V18" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W18" s="3" t="s">
+        <v>749</v>
+      </c>
+      <c r="X18" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="Y18" s="3" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="G19" s="6">
+        <v>28</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>752</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="J19" s="6">
+        <v>22</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>705</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="N19" s="6">
+        <v>47</v>
+      </c>
+      <c r="O19" s="6">
+        <v>47</v>
+      </c>
+      <c r="P19" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="R19" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S19" s="7" t="s">
+        <v>753</v>
+      </c>
+      <c r="T19" s="7" t="s">
+        <v>754</v>
+      </c>
+      <c r="U19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V19" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W19" s="7" t="s">
+        <v>755</v>
+      </c>
+      <c r="X19" s="7" t="s">
+        <v>756</v>
+      </c>
+      <c r="Y19" s="7" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>758</v>
+      </c>
+      <c r="G20" s="2">
+        <v>26</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>758</v>
+      </c>
+      <c r="J20" s="2">
+        <v>23</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>759</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>758</v>
+      </c>
+      <c r="N20" s="2">
+        <v>80</v>
+      </c>
+      <c r="O20" s="2">
+        <v>80</v>
+      </c>
+      <c r="P20" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="3" t="s">
+        <v>760</v>
+      </c>
+      <c r="R20" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S20" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="T20" s="3" t="s">
+        <v>762</v>
+      </c>
+      <c r="U20" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V20" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W20" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="X20" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="Y20" s="3" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="G21" s="9">
+        <v>11</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="J21" s="6">
+        <v>10</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="N21" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="O21" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P21" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="R21" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="S21" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="T21" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="U21" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="V21" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W21" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="X21" s="7" t="s">
+        <v>767</v>
+      </c>
+      <c r="Y21" s="7" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="G22" s="5">
+        <v>18</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>677</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="J22" s="2">
+        <v>16</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M22" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="N22" s="2">
+        <v>39</v>
+      </c>
+      <c r="O22" s="2">
+        <v>39</v>
+      </c>
+      <c r="P22" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="3" t="s">
+        <v>770</v>
+      </c>
+      <c r="R22" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="S22" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="T22" s="3" t="s">
+        <v>772</v>
+      </c>
+      <c r="U22" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V22" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W22" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="X22" s="3" t="s">
+        <v>774</v>
+      </c>
+      <c r="Y22" s="3" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="G23" s="9">
+        <v>16</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="J23" s="6">
+        <v>15</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="N23" s="6">
+        <v>26</v>
+      </c>
+      <c r="O23" s="6">
+        <v>26</v>
+      </c>
+      <c r="P23" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="7" t="s">
+        <v>776</v>
+      </c>
+      <c r="R23" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S23" s="7" t="s">
+        <v>777</v>
+      </c>
+      <c r="T23" s="7" t="s">
+        <v>778</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V23" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W23" s="7" t="s">
+        <v>779</v>
+      </c>
+      <c r="X23" s="7" t="s">
+        <v>780</v>
+      </c>
+      <c r="Y23" s="7" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="G24" s="5">
+        <v>5</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="J24" s="2">
+        <v>5</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="N24" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O24" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P24" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="R24" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="S24" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="T24" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="U24" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="V24" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W24" s="3" t="s">
+        <v>782</v>
+      </c>
+      <c r="X24" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="Y24" s="3" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="G25" s="9">
+        <v>3</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="J25" s="6">
+        <v>2</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="N25" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="O25" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P25" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="R25" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="S25" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="T25" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="U25" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="V25" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W25" s="7" t="s">
+        <v>785</v>
+      </c>
+      <c r="X25" s="7" t="s">
+        <v>786</v>
+      </c>
+      <c r="Y25" s="7" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="G26" s="5">
+        <v>2</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="J26" s="2">
+        <v>2</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="N26" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O26" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P26" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="R26" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="S26" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="T26" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="U26" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="V26" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W26" s="3" t="s">
+        <v>788</v>
+      </c>
+      <c r="X26" s="3" t="s">
+        <v>789</v>
+      </c>
+      <c r="Y26" s="3" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="G27" s="9">
+        <v>4</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="J27" s="6">
+        <v>4</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="M27" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="N27" s="6">
+        <v>11</v>
+      </c>
+      <c r="O27" s="6">
+        <v>11</v>
+      </c>
+      <c r="P27" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="7" t="s">
+        <v>791</v>
+      </c>
+      <c r="R27" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S27" s="7" t="s">
+        <v>792</v>
+      </c>
+      <c r="T27" s="7" t="s">
+        <v>793</v>
+      </c>
+      <c r="U27" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V27" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W27" s="7" t="s">
+        <v>794</v>
+      </c>
+      <c r="X27" s="7" t="s">
+        <v>795</v>
+      </c>
+      <c r="Y27" s="7" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="G28" s="5">
+        <v>3</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="J28" s="2">
+        <v>3</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M28" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="N28" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O28" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P28" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="R28" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="S28" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="T28" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="U28" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="V28" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W28" s="3" t="s">
+        <v>798</v>
+      </c>
+      <c r="X28" s="3" t="s">
+        <v>799</v>
+      </c>
+      <c r="Y28" s="3" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="G29" s="9">
+        <v>9</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="J29" s="6">
+        <v>8</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M29" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="N29" s="6">
+        <v>26</v>
+      </c>
+      <c r="O29" s="6">
+        <v>26</v>
+      </c>
+      <c r="P29" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="R29" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S29" s="7" t="s">
+        <v>802</v>
+      </c>
+      <c r="T29" s="7" t="s">
+        <v>803</v>
+      </c>
+      <c r="U29" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V29" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W29" s="7" t="s">
+        <v>804</v>
+      </c>
+      <c r="X29" s="7" t="s">
+        <v>805</v>
+      </c>
+      <c r="Y29" s="7" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="G30" s="5">
+        <v>4</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="J30" s="2">
+        <v>4</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="L30" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M30" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="N30" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O30" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P30" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="R30" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="S30" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="T30" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="U30" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="V30" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W30" s="3" t="s">
+        <v>807</v>
+      </c>
+      <c r="X30" s="3" t="s">
+        <v>808</v>
+      </c>
+      <c r="Y30" s="3" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="G31" s="9">
+        <v>18</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="J31" s="6">
+        <v>15</v>
+      </c>
+      <c r="K31" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="M31" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="N31" s="6">
+        <v>15</v>
+      </c>
+      <c r="O31" s="6">
+        <v>15</v>
+      </c>
+      <c r="P31" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="R31" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S31" s="7" t="s">
+        <v>810</v>
+      </c>
+      <c r="T31" s="7" t="s">
+        <v>811</v>
+      </c>
+      <c r="U31" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V31" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W31" s="7" t="s">
+        <v>812</v>
+      </c>
+      <c r="X31" s="7" t="s">
+        <v>813</v>
+      </c>
+      <c r="Y31" s="7" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G32" s="5">
+        <v>13</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="J32" s="2">
+        <v>12</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="L32" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="N32" s="2">
+        <v>45</v>
+      </c>
+      <c r="O32" s="2">
+        <v>45</v>
+      </c>
+      <c r="P32" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="R32" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S32" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="T32" s="3" t="s">
+        <v>816</v>
+      </c>
+      <c r="U32" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V32" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W32" s="3" t="s">
+        <v>817</v>
+      </c>
+      <c r="X32" s="3" t="s">
+        <v>818</v>
+      </c>
+      <c r="Y32" s="3" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="G33" s="9">
+        <v>6</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="J33" s="6">
+        <v>6</v>
+      </c>
+      <c r="K33" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="M33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="N33" s="6">
+        <v>19</v>
+      </c>
+      <c r="O33" s="6">
+        <v>19</v>
+      </c>
+      <c r="P33" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="R33" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S33" s="7" t="s">
+        <v>820</v>
+      </c>
+      <c r="T33" s="7" t="s">
+        <v>821</v>
+      </c>
+      <c r="U33" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V33" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W33" s="7" t="s">
+        <v>822</v>
+      </c>
+      <c r="X33" s="7" t="s">
+        <v>823</v>
+      </c>
+      <c r="Y33" s="7" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="G34" s="5">
+        <v>12</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="J34" s="2">
+        <v>11</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>825</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M34" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="N34" s="2">
+        <v>12</v>
+      </c>
+      <c r="O34" s="2">
+        <v>12</v>
+      </c>
+      <c r="P34" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="R34" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S34" s="3" t="s">
+        <v>826</v>
+      </c>
+      <c r="T34" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="U34" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V34" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W34" s="3" t="s">
+        <v>827</v>
+      </c>
+      <c r="X34" s="3" t="s">
+        <v>828</v>
+      </c>
+      <c r="Y34" s="3" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="G35" s="11">
+        <v>14</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="J35" s="6">
+        <v>12</v>
+      </c>
+      <c r="K35" s="7" t="s">
+        <v>830</v>
+      </c>
+      <c r="L35" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M35" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="N35" s="6">
+        <v>14</v>
+      </c>
+      <c r="O35" s="6">
+        <v>14</v>
+      </c>
+      <c r="P35" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="R35" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S35" s="7" t="s">
+        <v>831</v>
+      </c>
+      <c r="T35" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="U35" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V35" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W35" s="7" t="s">
+        <v>832</v>
+      </c>
+      <c r="X35" s="7" t="s">
+        <v>833</v>
+      </c>
+      <c r="Y35" s="7" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="G36" s="5">
+        <v>8</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="J36" s="2">
+        <v>7</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="N36" s="2">
+        <v>7</v>
+      </c>
+      <c r="O36" s="2">
+        <v>7</v>
+      </c>
+      <c r="P36" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R36" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S36" s="3" t="s">
+        <v>835</v>
+      </c>
+      <c r="T36" s="3" t="s">
+        <v>836</v>
+      </c>
+      <c r="U36" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V36" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W36" s="3" t="s">
+        <v>837</v>
+      </c>
+      <c r="X36" s="3" t="s">
+        <v>838</v>
+      </c>
+      <c r="Y36" s="3" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="G37" s="9">
+        <v>10</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="J37" s="6">
+        <v>9</v>
+      </c>
+      <c r="K37" s="7" t="s">
+        <v>840</v>
+      </c>
+      <c r="L37" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M37" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="N37" s="6">
+        <v>42</v>
+      </c>
+      <c r="O37" s="6">
+        <v>42</v>
+      </c>
+      <c r="P37" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="R37" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S37" s="7" t="s">
+        <v>841</v>
+      </c>
+      <c r="T37" s="7" t="s">
+        <v>842</v>
+      </c>
+      <c r="U37" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V37" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W37" s="7" t="s">
+        <v>843</v>
+      </c>
+      <c r="X37" s="7" t="s">
+        <v>844</v>
+      </c>
+      <c r="Y37" s="7" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="G38" s="5">
+        <v>4</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="J38" s="2">
+        <v>5</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="M38" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="N38" s="2">
+        <v>7</v>
+      </c>
+      <c r="O38" s="2">
+        <v>7</v>
+      </c>
+      <c r="P38" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="3" t="s">
+        <v>846</v>
+      </c>
+      <c r="R38" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S38" s="3" t="s">
+        <v>847</v>
+      </c>
+      <c r="T38" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="U38" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V38" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W38" s="3" t="s">
+        <v>848</v>
+      </c>
+      <c r="X38" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="Y38" s="3" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="G39" s="9">
+        <v>10</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="J39" s="6">
+        <v>9</v>
+      </c>
+      <c r="K39" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="L39" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M39" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="N39" s="6">
+        <v>11</v>
+      </c>
+      <c r="O39" s="6">
+        <v>11</v>
+      </c>
+      <c r="P39" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="R39" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S39" s="7" t="s">
+        <v>851</v>
+      </c>
+      <c r="T39" s="7" t="s">
+        <v>852</v>
+      </c>
+      <c r="U39" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V39" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W39" s="7" t="s">
+        <v>853</v>
+      </c>
+      <c r="X39" s="7" t="s">
+        <v>854</v>
+      </c>
+      <c r="Y39" s="7" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="G40" s="5">
+        <v>3</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="J40" s="2">
+        <v>3</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="L40" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M40" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="N40" s="2">
+        <v>3</v>
+      </c>
+      <c r="O40" s="2">
+        <v>3</v>
+      </c>
+      <c r="P40" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="R40" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S40" s="3" t="s">
+        <v>856</v>
+      </c>
+      <c r="T40" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="U40" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V40" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W40" s="3" t="s">
+        <v>857</v>
+      </c>
+      <c r="X40" s="3" t="s">
+        <v>858</v>
+      </c>
+      <c r="Y40" s="3" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="G41" s="9">
+        <v>5</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="J41" s="6">
+        <v>5</v>
+      </c>
+      <c r="K41" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="L41" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="M41" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="N41" s="6">
+        <v>5</v>
+      </c>
+      <c r="O41" s="6">
+        <v>5</v>
+      </c>
+      <c r="P41" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="R41" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S41" s="7" t="s">
+        <v>860</v>
+      </c>
+      <c r="T41" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="U41" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V41" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W41" s="7" t="s">
+        <v>861</v>
+      </c>
+      <c r="X41" s="7" t="s">
+        <v>862</v>
+      </c>
+      <c r="Y41" s="7" t="s">
+        <v>863</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Y1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto-collected traffic data: 2026-09-03 07:15 PM IST [07_00 PM]
</commit_message>
<xml_diff>
--- a/output/excel/Kolkata_Traffic_Data_2026-09-03.xlsx
+++ b/output/excel/Kolkata_Traffic_Data_2026-09-03.xlsx
@@ -7,13 +7,14 @@
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="01_00 PM" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="07_00 PM" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2501" uniqueCount="864">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3326" uniqueCount="1058">
   <si>
     <t>Route ID</t>
   </si>
@@ -2852,6 +2853,677 @@
   </si>
   <si>
     <t>screenshots/2026-09-03/01_00 PM/S19_Bagha_Jatin___Baishnabghata/bus.jpg</t>
+  </si>
+  <si>
+    <t>07_00 PM</t>
+  </si>
+  <si>
+    <t>Thursday (Weekday) - 07_00 PM</t>
+  </si>
+  <si>
+    <t>0.87x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M01_DH_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M01_DH_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M01_DH_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 min
+7:15 AM—7:36 AM
+S-185</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M02_B_T_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M02_B_T_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M02_B_T_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>23.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43 min
+7:11 AM—7:54 AM
+Barrackpore Chiriamore - Salap More
+7:11 AM from Dunlop More
+Details</t>
+  </si>
+  <si>
+    <t>1.39x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M03_B_T_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M03_B_T_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M03_B_T_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>11.8</t>
+  </si>
+  <si>
+    <t>-12 min (Bike Faster)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32 min
+7:20 AM—7:52 AM
+L238
+7:20 AM from Muchi Bazar
+Details</t>
+  </si>
+  <si>
+    <t>0.46x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M04_VIP_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M04_VIP_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M04_VIP_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>11.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38 min
+7:33 AM—8:11 AM
+79B</t>
+  </si>
+  <si>
+    <t>0.63x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M05_Jessore_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M05_Jessore_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M05_Jessore_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 min
+7:09 AM—7:26 AM
+DN-9/1</t>
+  </si>
+  <si>
+    <t>0.65x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M06_Airport_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M06_Airport_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M06_Airport_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>10.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28 min
+7:10 AM—7:38 AM
+230</t>
+  </si>
+  <si>
+    <t>0.61x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M07_APC_Bose_Rd/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M07_APC_Bose_Rd/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M07_APC_Bose_Rd/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 min
+7:09 AM—7:31 AM
+  47B</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M08_Bidhan_Sarani/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M08_Bidhan_Sarani/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M08_Bidhan_Sarani/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 min
+7:13 AM—7:30 AM
+214A</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M09_Central_Avenue__C_R_Avenue_/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M09_Central_Avenue__C_R_Avenue_/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M09_Central_Avenue__C_R_Avenue_/bus.jpg</t>
+  </si>
+  <si>
+    <t>7.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 min
+7:08 AM—7:15 AM
+S-12N</t>
+  </si>
+  <si>
+    <t>0.37x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M10_S_N_Banerjee_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M10_S_N_Banerjee_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M10_S_N_Banerjee_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>9.0</t>
+  </si>
+  <si>
+    <t>11.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+7:13 AM—7:26 AM
+24</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M11_M_G_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M11_M_G_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M11_M_G_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 min
+7:13 AM—7:21 AM
+240</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M12_C_I_T_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M12_C_I_T_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M12_C_I_T_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>10.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+7:07 AM—7:20 AM
+221
+7:07 AM from AJC Bose Road
+Details</t>
+  </si>
+  <si>
+    <t>0.48x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M13_Sarat_Bose_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M13_Sarat_Bose_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M13_Sarat_Bose_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>16.8 km</t>
+  </si>
+  <si>
+    <t>11.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 hr
+7:05 AM—8:05 AM
+222  S-112</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M14_S_P_Mukherjee_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M14_S_P_Mukherjee_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M14_S_P_Mukherjee_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19 min
+7:28 AM—7:47 AM
+42A  18C</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M15_Hazra_Road___S_P_Mukherjee_Road_connector/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M15_Hazra_Road___S_P_Mukherjee_Road_connector/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M15_Hazra_Road___S_P_Mukherjee_Road_connector/bus.jpg</t>
+  </si>
+  <si>
+    <t>8.7</t>
+  </si>
+  <si>
+    <t>10.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 min
+7:27 AM—7:37 AM
+M-14</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M16_Gariahat_Road___Rashbehari_Avenue/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M16_Gariahat_Road___Rashbehari_Avenue/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M16_Gariahat_Road___Rashbehari_Avenue/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 min
+7:33 AM—7:42 AM
+S-22</t>
+  </si>
+  <si>
+    <t>0.53x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M18_Chetla_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M18_Chetla_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M18_Chetla_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+7:24 AM—7:37 AM
+SD5</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M19_Taratala_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M19_Taratala_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M19_Taratala_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 min
+7:01 AM—7:25 AM
+ST-6
+7:01 AM from Tollygunge Metro
+Details</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M20_Prince_Anwar_Shah_Rd/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M20_Prince_Anwar_Shah_Rd/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M20_Prince_Anwar_Shah_Rd/bus.jpg</t>
+  </si>
+  <si>
+    <t>16.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 min
+7:18 AM—7:28 AM
+S-9</t>
+  </si>
+  <si>
+    <t>0.77x</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M21_Karunamoyee_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M21_Karunamoyee_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M21_Karunamoyee_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>13.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 min
+7:19 AM—7:34 AM
+S-22</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M22_Canal_South_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M22_Canal_South_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M22_Canal_South_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t>13.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 min
+7:10 AM—7:23 AM
+Berachampa - Karunamoyee</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M23_VIP_Road_connector/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M23_VIP_Road_connector/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/M23_VIP_Road_connector/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 min
+7:10 AM—7:14 AM
+Kamal Gazi Bypass - Dankuni Housing</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S01_Baishnabghata_Patuli/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S01_Baishnabghata_Patuli/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S01_Baishnabghata_Patuli/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 min
+7:05 AM—7:09 AM
+AC-24A</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S02_Patuli___Highland_Park/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S02_Patuli___Highland_Park/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S02_Patuli___Highland_Park/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 min
+7:09 AM—7:12 AM
+AC-24A</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S03_Highland_Park___Ajaynagar/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S03_Highland_Park___Ajaynagar/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S03_Highland_Park___Ajaynagar/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 min
+7:12 AM—7:18 AM
+S-21</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S04_Ajaynagar___Kalikapur/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S04_Ajaynagar___Kalikapur/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S04_Ajaynagar___Kalikapur/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 min
+7:02 AM—7:06 AM
+Barasat - Baruipur</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S05_Kalikapur___Ruby/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S05_Kalikapur___Ruby/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S05_Kalikapur___Ruby/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 min
+7:24 AM—7:38 AM
+Garia No. 6 - Ultadanga</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S06_Ruby___Science_City/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S06_Ruby___Science_City/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S06_Ruby___Science_City/bus.jpg</t>
+  </si>
+  <si>
+    <t>1.8 km</t>
+  </si>
+  <si>
+    <t>21.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 min
+7:11 AM—7:16 AM
+Ecospace Amity University - Andul Station Road</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S07_Science_City___Chingrighata/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S07_Science_City___Chingrighata/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S07_Science_City___Chingrighata/bus.jpg</t>
+  </si>
+  <si>
+    <t>13.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 min
+7:27 AM—7:42 AM
+S-12N</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S08_Chingrighata___Sealdah/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S08_Chingrighata___Sealdah/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S08_Chingrighata___Sealdah/bus.jpg</t>
+  </si>
+  <si>
+    <t>9.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 min
+7:00 AM—7:18 AM
+DN-17  240  </t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S09_Sealdah___Park_Circus/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S09_Sealdah___Park_Circus/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S09_Sealdah___Park_Circus/bus.jpg</t>
+  </si>
+  <si>
+    <t>32.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19 min
+7:40 AM—7:59 AM
+EB-14  </t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S10_Park_Circus___Science_City/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S10_Park_Circus___Science_City/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S10_Park_Circus___Science_City/bus.jpg</t>
+  </si>
+  <si>
+    <t>10.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 min
+7:01 AM—7:10 AM
+45A
+7:02 AM from Zeeshan
+ 1 min
+Details</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S11_Park_Circus___Gariahat/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S11_Park_Circus___Gariahat/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S11_Park_Circus___Gariahat/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 min
+7:14 AM—7:28 AM
+Barasat - Botanical Garden</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S12_Gariahat___Ruby/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S12_Gariahat___Ruby/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S12_Gariahat___Ruby/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 min
+7:12 AM—7:19 AM
+45</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S13_Gariahat___Mallick_Road/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S13_Gariahat___Mallick_Road/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S13_Gariahat___Mallick_Road/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 min
+7:28 AM—7:39 AM
+Cityflo</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S14_Jadavpur_Police_St____Kalikapur/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S14_Jadavpur_Police_St____Kalikapur/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S14_Jadavpur_Police_St____Kalikapur/bus.jpg</t>
+  </si>
+  <si>
+    <t>13.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 min
+7:13 AM—7:18 AM
+S-31</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S15_Mallick_Road___Jadavpur_Sulekha/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S15_Mallick_Road___Jadavpur_Sulekha/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S15_Mallick_Road___Jadavpur_Sulekha/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 min
+7:09 AM—7:19 AM
+S-9</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S16_Jadavpur_Sulekha___Ajay_Nagar/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S16_Jadavpur_Sulekha___Ajay_Nagar/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S16_Jadavpur_Sulekha___Ajay_Nagar/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 min
+7:20 AM—7:23 AM
+S-5</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S17_Jadavpur_Sulekha___Bagha_Jatin/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S17_Jadavpur_Sulekha___Bagha_Jatin/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S17_Jadavpur_Sulekha___Bagha_Jatin/bus.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 min
+7:27 AM—7:32 AM
+45</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S19_Bagha_Jatin___Baishnabghata/car.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S19_Bagha_Jatin___Baishnabghata/bike.jpg</t>
+  </si>
+  <si>
+    <t>screenshots/2026-09-03/07_00 PM/S19_Bagha_Jatin___Baishnabghata/bus.jpg</t>
   </si>
 </sst>
 </file>
@@ -2957,7 +3629,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2990,6 +3662,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -12905,6 +13580,3199 @@
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Y41"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="33" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="25" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="29" customWidth="1"/>
+    <col min="16" max="16" width="30" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="18" max="18" width="21" customWidth="1"/>
+    <col min="19" max="19" width="45" customWidth="1"/>
+    <col min="20" max="20" width="20" customWidth="1"/>
+    <col min="21" max="21" width="23" customWidth="1"/>
+    <col min="22" max="25" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="2">
+        <v>79</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J2" s="2">
+        <v>70</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N2" s="2">
+        <v>69</v>
+      </c>
+      <c r="O2" s="2">
+        <v>69</v>
+      </c>
+      <c r="P2" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>867</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>868</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="6">
+        <v>28</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>659</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3" s="6">
+        <v>24</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>549</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="N3" s="6">
+        <v>21</v>
+      </c>
+      <c r="O3" s="6">
+        <v>21</v>
+      </c>
+      <c r="P3" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S3" s="7" t="s">
+        <v>870</v>
+      </c>
+      <c r="T3" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="U3" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V3" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W3" s="7" t="s">
+        <v>871</v>
+      </c>
+      <c r="X3" s="7" t="s">
+        <v>872</v>
+      </c>
+      <c r="Y3" s="7" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="2">
+        <v>31</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>874</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="2">
+        <v>30</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="N4" s="2">
+        <v>43</v>
+      </c>
+      <c r="O4" s="2">
+        <v>43</v>
+      </c>
+      <c r="P4" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>875</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>876</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W4" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="X4" s="3" t="s">
+        <v>878</v>
+      </c>
+      <c r="Y4" s="3" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="G5" s="6">
+        <v>70</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>880</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="J5" s="6">
+        <v>58</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>881</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="N5" s="6">
+        <v>32</v>
+      </c>
+      <c r="O5" s="6">
+        <v>32</v>
+      </c>
+      <c r="P5" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="R5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S5" s="7" t="s">
+        <v>882</v>
+      </c>
+      <c r="T5" s="7" t="s">
+        <v>883</v>
+      </c>
+      <c r="U5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V5" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W5" s="7" t="s">
+        <v>884</v>
+      </c>
+      <c r="X5" s="7" t="s">
+        <v>885</v>
+      </c>
+      <c r="Y5" s="7" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G6" s="2">
+        <v>60</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>887</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="2">
+        <v>49</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>706</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="N6" s="2">
+        <v>38</v>
+      </c>
+      <c r="O6" s="2">
+        <v>38</v>
+      </c>
+      <c r="P6" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S6" s="3" t="s">
+        <v>888</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="U6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V6" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W6" s="3" t="s">
+        <v>890</v>
+      </c>
+      <c r="X6" s="3" t="s">
+        <v>891</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G7" s="6">
+        <v>26</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>846</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="J7" s="6">
+        <v>20</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="N7" s="6">
+        <v>17</v>
+      </c>
+      <c r="O7" s="6">
+        <v>17</v>
+      </c>
+      <c r="P7" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S7" s="7" t="s">
+        <v>893</v>
+      </c>
+      <c r="T7" s="7" t="s">
+        <v>894</v>
+      </c>
+      <c r="U7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V7" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W7" s="7" t="s">
+        <v>895</v>
+      </c>
+      <c r="X7" s="7" t="s">
+        <v>896</v>
+      </c>
+      <c r="Y7" s="7" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G8" s="5">
+        <v>46</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>898</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="J8" s="2">
+        <v>40</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="N8" s="2">
+        <v>28</v>
+      </c>
+      <c r="O8" s="2">
+        <v>28</v>
+      </c>
+      <c r="P8" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S8" s="3" t="s">
+        <v>899</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>900</v>
+      </c>
+      <c r="U8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V8" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W8" s="3" t="s">
+        <v>901</v>
+      </c>
+      <c r="X8" s="3" t="s">
+        <v>902</v>
+      </c>
+      <c r="Y8" s="3" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="G9" s="6">
+        <v>31</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>495</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="J9" s="6">
+        <v>28</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>480</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="N9" s="6">
+        <v>22</v>
+      </c>
+      <c r="O9" s="6">
+        <v>22</v>
+      </c>
+      <c r="P9" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S9" s="7" t="s">
+        <v>904</v>
+      </c>
+      <c r="T9" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="U9" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V9" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W9" s="7" t="s">
+        <v>905</v>
+      </c>
+      <c r="X9" s="7" t="s">
+        <v>906</v>
+      </c>
+      <c r="Y9" s="7" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G10" s="2">
+        <v>27</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>846</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="J10" s="2">
+        <v>25</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="N10" s="2">
+        <v>17</v>
+      </c>
+      <c r="O10" s="2">
+        <v>17</v>
+      </c>
+      <c r="P10" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="R10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S10" s="3" t="s">
+        <v>908</v>
+      </c>
+      <c r="T10" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="U10" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V10" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W10" s="3" t="s">
+        <v>909</v>
+      </c>
+      <c r="X10" s="3" t="s">
+        <v>910</v>
+      </c>
+      <c r="Y10" s="3" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G11" s="6">
+        <v>19</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>912</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="J11" s="6">
+        <v>15</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="N11" s="6">
+        <v>7</v>
+      </c>
+      <c r="O11" s="6">
+        <v>7</v>
+      </c>
+      <c r="P11" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S11" s="7" t="s">
+        <v>913</v>
+      </c>
+      <c r="T11" s="7" t="s">
+        <v>914</v>
+      </c>
+      <c r="U11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V11" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W11" s="7" t="s">
+        <v>915</v>
+      </c>
+      <c r="X11" s="7" t="s">
+        <v>916</v>
+      </c>
+      <c r="Y11" s="7" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="G12" s="2">
+        <v>28</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>918</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="J12" s="2">
+        <v>23</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>919</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="N12" s="2">
+        <v>13</v>
+      </c>
+      <c r="O12" s="2">
+        <v>13</v>
+      </c>
+      <c r="P12" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="R12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S12" s="3" t="s">
+        <v>920</v>
+      </c>
+      <c r="T12" s="3" t="s">
+        <v>883</v>
+      </c>
+      <c r="U12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V12" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W12" s="3" t="s">
+        <v>921</v>
+      </c>
+      <c r="X12" s="3" t="s">
+        <v>922</v>
+      </c>
+      <c r="Y12" s="3" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="G13" s="9">
+        <v>13</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="J13" s="6">
+        <v>11</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>717</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="N13" s="6">
+        <v>8</v>
+      </c>
+      <c r="O13" s="6">
+        <v>8</v>
+      </c>
+      <c r="P13" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S13" s="7" t="s">
+        <v>924</v>
+      </c>
+      <c r="T13" s="7" t="s">
+        <v>690</v>
+      </c>
+      <c r="U13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V13" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W13" s="7" t="s">
+        <v>925</v>
+      </c>
+      <c r="X13" s="7" t="s">
+        <v>926</v>
+      </c>
+      <c r="Y13" s="7" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G14" s="2">
+        <v>27</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>752</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="J14" s="2">
+        <v>22</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>928</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="N14" s="2">
+        <v>13</v>
+      </c>
+      <c r="O14" s="2">
+        <v>13</v>
+      </c>
+      <c r="P14" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="R14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S14" s="3" t="s">
+        <v>929</v>
+      </c>
+      <c r="T14" s="3" t="s">
+        <v>930</v>
+      </c>
+      <c r="U14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V14" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W14" s="3" t="s">
+        <v>931</v>
+      </c>
+      <c r="X14" s="3" t="s">
+        <v>932</v>
+      </c>
+      <c r="Y14" s="3" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>934</v>
+      </c>
+      <c r="G15" s="6">
+        <v>85</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>935</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>934</v>
+      </c>
+      <c r="J15" s="6">
+        <v>73</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>881</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>934</v>
+      </c>
+      <c r="N15" s="6">
+        <v>60</v>
+      </c>
+      <c r="O15" s="6">
+        <v>60</v>
+      </c>
+      <c r="P15" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S15" s="7" t="s">
+        <v>936</v>
+      </c>
+      <c r="T15" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V15" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W15" s="7" t="s">
+        <v>937</v>
+      </c>
+      <c r="X15" s="7" t="s">
+        <v>938</v>
+      </c>
+      <c r="Y15" s="7" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="G16" s="2">
+        <v>31</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>734</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="J16" s="2">
+        <v>25</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>919</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="N16" s="2">
+        <v>19</v>
+      </c>
+      <c r="O16" s="2">
+        <v>19</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="R16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S16" s="3" t="s">
+        <v>940</v>
+      </c>
+      <c r="T16" s="3" t="s">
+        <v>900</v>
+      </c>
+      <c r="U16" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V16" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W16" s="3" t="s">
+        <v>941</v>
+      </c>
+      <c r="X16" s="3" t="s">
+        <v>942</v>
+      </c>
+      <c r="Y16" s="3" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="G17" s="6">
+        <v>20</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>944</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J17" s="6">
+        <v>17</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>945</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="N17" s="6">
+        <v>10</v>
+      </c>
+      <c r="O17" s="6">
+        <v>10</v>
+      </c>
+      <c r="P17" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="R17" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S17" s="7" t="s">
+        <v>946</v>
+      </c>
+      <c r="T17" s="7" t="s">
+        <v>713</v>
+      </c>
+      <c r="U17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V17" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W17" s="7" t="s">
+        <v>947</v>
+      </c>
+      <c r="X17" s="7" t="s">
+        <v>948</v>
+      </c>
+      <c r="Y17" s="7" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="G18" s="2">
+        <v>17</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="J18" s="2">
+        <v>13</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>659</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="N18" s="2">
+        <v>9</v>
+      </c>
+      <c r="O18" s="2">
+        <v>9</v>
+      </c>
+      <c r="P18" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="3" t="s">
+        <v>524</v>
+      </c>
+      <c r="R18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S18" s="3" t="s">
+        <v>950</v>
+      </c>
+      <c r="T18" s="3" t="s">
+        <v>951</v>
+      </c>
+      <c r="U18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V18" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W18" s="3" t="s">
+        <v>952</v>
+      </c>
+      <c r="X18" s="3" t="s">
+        <v>953</v>
+      </c>
+      <c r="Y18" s="3" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="G19" s="6">
+        <v>21</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="J19" s="6">
+        <v>19</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="N19" s="6">
+        <v>13</v>
+      </c>
+      <c r="O19" s="6">
+        <v>13</v>
+      </c>
+      <c r="P19" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="R19" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S19" s="7" t="s">
+        <v>955</v>
+      </c>
+      <c r="T19" s="7" t="s">
+        <v>690</v>
+      </c>
+      <c r="U19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V19" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W19" s="7" t="s">
+        <v>956</v>
+      </c>
+      <c r="X19" s="7" t="s">
+        <v>957</v>
+      </c>
+      <c r="Y19" s="7" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="G20" s="5">
+        <v>29</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="J20" s="2">
+        <v>27</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="N20" s="2">
+        <v>24</v>
+      </c>
+      <c r="O20" s="2">
+        <v>24</v>
+      </c>
+      <c r="P20" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="R20" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S20" s="3" t="s">
+        <v>959</v>
+      </c>
+      <c r="T20" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="U20" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V20" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W20" s="3" t="s">
+        <v>960</v>
+      </c>
+      <c r="X20" s="3" t="s">
+        <v>961</v>
+      </c>
+      <c r="Y20" s="3" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="G21" s="9">
+        <v>13</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="J21" s="6">
+        <v>12</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>963</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="N21" s="6">
+        <v>10</v>
+      </c>
+      <c r="O21" s="6">
+        <v>10</v>
+      </c>
+      <c r="P21" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="R21" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S21" s="7" t="s">
+        <v>964</v>
+      </c>
+      <c r="T21" s="7" t="s">
+        <v>965</v>
+      </c>
+      <c r="U21" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V21" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W21" s="7" t="s">
+        <v>966</v>
+      </c>
+      <c r="X21" s="7" t="s">
+        <v>967</v>
+      </c>
+      <c r="Y21" s="7" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="G22" s="2">
+        <v>25</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>969</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="J22" s="2">
+        <v>21</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="M22" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="N22" s="2">
+        <v>15</v>
+      </c>
+      <c r="O22" s="2">
+        <v>15</v>
+      </c>
+      <c r="P22" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="R22" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S22" s="3" t="s">
+        <v>970</v>
+      </c>
+      <c r="T22" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="U22" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V22" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W22" s="3" t="s">
+        <v>971</v>
+      </c>
+      <c r="X22" s="3" t="s">
+        <v>972</v>
+      </c>
+      <c r="Y22" s="3" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="G23" s="6">
+        <v>21</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="J23" s="6">
+        <v>19</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>974</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="N23" s="6">
+        <v>13</v>
+      </c>
+      <c r="O23" s="6">
+        <v>13</v>
+      </c>
+      <c r="P23" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="R23" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S23" s="7" t="s">
+        <v>975</v>
+      </c>
+      <c r="T23" s="7" t="s">
+        <v>690</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V23" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W23" s="7" t="s">
+        <v>976</v>
+      </c>
+      <c r="X23" s="7" t="s">
+        <v>977</v>
+      </c>
+      <c r="Y23" s="7" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="G24" s="5">
+        <v>6</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="J24" s="2">
+        <v>6</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="N24" s="2">
+        <v>4</v>
+      </c>
+      <c r="O24" s="2">
+        <v>4</v>
+      </c>
+      <c r="P24" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="R24" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S24" s="3" t="s">
+        <v>979</v>
+      </c>
+      <c r="T24" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="U24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V24" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W24" s="3" t="s">
+        <v>980</v>
+      </c>
+      <c r="X24" s="3" t="s">
+        <v>981</v>
+      </c>
+      <c r="Y24" s="3" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="G25" s="9">
+        <v>3</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="J25" s="6">
+        <v>2</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="N25" s="6">
+        <v>4</v>
+      </c>
+      <c r="O25" s="6">
+        <v>4</v>
+      </c>
+      <c r="P25" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="R25" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S25" s="7" t="s">
+        <v>983</v>
+      </c>
+      <c r="T25" s="7" t="s">
+        <v>568</v>
+      </c>
+      <c r="U25" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V25" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W25" s="7" t="s">
+        <v>984</v>
+      </c>
+      <c r="X25" s="7" t="s">
+        <v>985</v>
+      </c>
+      <c r="Y25" s="7" t="s">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="G26" s="5">
+        <v>2</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="J26" s="2">
+        <v>2</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="N26" s="2">
+        <v>3</v>
+      </c>
+      <c r="O26" s="2">
+        <v>3</v>
+      </c>
+      <c r="P26" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="R26" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S26" s="3" t="s">
+        <v>987</v>
+      </c>
+      <c r="T26" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="U26" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V26" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W26" s="3" t="s">
+        <v>988</v>
+      </c>
+      <c r="X26" s="3" t="s">
+        <v>989</v>
+      </c>
+      <c r="Y26" s="3" t="s">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="G27" s="9">
+        <v>4</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="J27" s="6">
+        <v>4</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="M27" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="N27" s="6">
+        <v>6</v>
+      </c>
+      <c r="O27" s="6">
+        <v>6</v>
+      </c>
+      <c r="P27" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="R27" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S27" s="7" t="s">
+        <v>991</v>
+      </c>
+      <c r="T27" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="U27" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V27" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W27" s="7" t="s">
+        <v>992</v>
+      </c>
+      <c r="X27" s="7" t="s">
+        <v>993</v>
+      </c>
+      <c r="Y27" s="7" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="G28" s="5">
+        <v>5</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="J28" s="2">
+        <v>4</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M28" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="N28" s="2">
+        <v>4</v>
+      </c>
+      <c r="O28" s="2">
+        <v>4</v>
+      </c>
+      <c r="P28" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="R28" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S28" s="3" t="s">
+        <v>995</v>
+      </c>
+      <c r="T28" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="U28" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V28" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W28" s="3" t="s">
+        <v>996</v>
+      </c>
+      <c r="X28" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="Y28" s="3" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="G29" s="6">
+        <v>13</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>513</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="J29" s="6">
+        <v>11</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>584</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M29" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="N29" s="6">
+        <v>14</v>
+      </c>
+      <c r="O29" s="6">
+        <v>14</v>
+      </c>
+      <c r="P29" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="R29" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S29" s="7" t="s">
+        <v>999</v>
+      </c>
+      <c r="T29" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="U29" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V29" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W29" s="7" t="s">
+        <v>1000</v>
+      </c>
+      <c r="X29" s="7" t="s">
+        <v>1001</v>
+      </c>
+      <c r="Y29" s="7" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>1003</v>
+      </c>
+      <c r="G30" s="2">
+        <v>5</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>1004</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>1003</v>
+      </c>
+      <c r="J30" s="2">
+        <v>4</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="L30" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M30" s="3" t="s">
+        <v>1003</v>
+      </c>
+      <c r="N30" s="2">
+        <v>5</v>
+      </c>
+      <c r="O30" s="2">
+        <v>5</v>
+      </c>
+      <c r="P30" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="3" t="s">
+        <v>1004</v>
+      </c>
+      <c r="R30" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S30" s="3" t="s">
+        <v>1005</v>
+      </c>
+      <c r="T30" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="U30" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V30" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W30" s="3" t="s">
+        <v>1006</v>
+      </c>
+      <c r="X30" s="3" t="s">
+        <v>1007</v>
+      </c>
+      <c r="Y30" s="3" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="G31" s="6">
+        <v>21</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>1009</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="J31" s="6">
+        <v>18</v>
+      </c>
+      <c r="K31" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="M31" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="N31" s="6">
+        <v>15</v>
+      </c>
+      <c r="O31" s="6">
+        <v>15</v>
+      </c>
+      <c r="P31" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="R31" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S31" s="7" t="s">
+        <v>1010</v>
+      </c>
+      <c r="T31" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="U31" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V31" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W31" s="7" t="s">
+        <v>1011</v>
+      </c>
+      <c r="X31" s="7" t="s">
+        <v>1012</v>
+      </c>
+      <c r="Y31" s="7" t="s">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G32" s="12">
+        <v>18</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>1014</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="J32" s="2">
+        <v>12</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="L32" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="M32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="N32" s="2">
+        <v>18</v>
+      </c>
+      <c r="O32" s="2">
+        <v>18</v>
+      </c>
+      <c r="P32" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="3" t="s">
+        <v>1014</v>
+      </c>
+      <c r="R32" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S32" s="3" t="s">
+        <v>1015</v>
+      </c>
+      <c r="T32" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="U32" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V32" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W32" s="3" t="s">
+        <v>1016</v>
+      </c>
+      <c r="X32" s="3" t="s">
+        <v>1017</v>
+      </c>
+      <c r="Y32" s="3" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="G33" s="6">
+        <v>6</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="J33" s="6">
+        <v>7</v>
+      </c>
+      <c r="K33" s="7" t="s">
+        <v>1019</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="M33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="N33" s="6">
+        <v>19</v>
+      </c>
+      <c r="O33" s="6">
+        <v>19</v>
+      </c>
+      <c r="P33" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="R33" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S33" s="7" t="s">
+        <v>1020</v>
+      </c>
+      <c r="T33" s="7" t="s">
+        <v>821</v>
+      </c>
+      <c r="U33" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V33" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="W33" s="7" t="s">
+        <v>1021</v>
+      </c>
+      <c r="X33" s="7" t="s">
+        <v>1022</v>
+      </c>
+      <c r="Y33" s="7" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="G34" s="5">
+        <v>15</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="J34" s="2">
+        <v>13</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M34" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="N34" s="2">
+        <v>9</v>
+      </c>
+      <c r="O34" s="2">
+        <v>9</v>
+      </c>
+      <c r="P34" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="R34" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="S34" s="3" t="s">
+        <v>1025</v>
+      </c>
+      <c r="T34" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="U34" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V34" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W34" s="3" t="s">
+        <v>1026</v>
+      </c>
+      <c r="X34" s="3" t="s">
+        <v>1027</v>
+      </c>
+      <c r="Y34" s="3" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="G35" s="11">
+        <v>17</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>555</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="J35" s="6">
+        <v>15</v>
+      </c>
+      <c r="K35" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="L35" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M35" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="N35" s="6">
+        <v>14</v>
+      </c>
+      <c r="O35" s="6">
+        <v>14</v>
+      </c>
+      <c r="P35" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="R35" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S35" s="7" t="s">
+        <v>1029</v>
+      </c>
+      <c r="T35" s="7" t="s">
+        <v>673</v>
+      </c>
+      <c r="U35" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V35" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W35" s="7" t="s">
+        <v>1030</v>
+      </c>
+      <c r="X35" s="7" t="s">
+        <v>1031</v>
+      </c>
+      <c r="Y35" s="7" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="G36" s="12">
+        <v>11</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="J36" s="2">
+        <v>10</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="N36" s="2">
+        <v>7</v>
+      </c>
+      <c r="O36" s="2">
+        <v>7</v>
+      </c>
+      <c r="P36" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R36" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S36" s="3" t="s">
+        <v>1033</v>
+      </c>
+      <c r="T36" s="3" t="s">
+        <v>613</v>
+      </c>
+      <c r="U36" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V36" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W36" s="3" t="s">
+        <v>1034</v>
+      </c>
+      <c r="X36" s="3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="Y36" s="3" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="G37" s="9">
+        <v>12</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="J37" s="6">
+        <v>11</v>
+      </c>
+      <c r="K37" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L37" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M37" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="N37" s="6">
+        <v>11</v>
+      </c>
+      <c r="O37" s="6">
+        <v>11</v>
+      </c>
+      <c r="P37" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="R37" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S37" s="7" t="s">
+        <v>1037</v>
+      </c>
+      <c r="T37" s="7" t="s">
+        <v>541</v>
+      </c>
+      <c r="U37" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V37" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W37" s="7" t="s">
+        <v>1038</v>
+      </c>
+      <c r="X37" s="7" t="s">
+        <v>1039</v>
+      </c>
+      <c r="Y37" s="7" t="s">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="G38" s="5">
+        <v>6</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>1041</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="J38" s="2">
+        <v>5</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M38" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="N38" s="2">
+        <v>5</v>
+      </c>
+      <c r="O38" s="2">
+        <v>5</v>
+      </c>
+      <c r="P38" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="R38" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S38" s="3" t="s">
+        <v>1042</v>
+      </c>
+      <c r="T38" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="U38" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V38" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W38" s="3" t="s">
+        <v>1043</v>
+      </c>
+      <c r="X38" s="3" t="s">
+        <v>1044</v>
+      </c>
+      <c r="Y38" s="3" t="s">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="G39" s="6">
+        <v>16</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>611</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="J39" s="6">
+        <v>10</v>
+      </c>
+      <c r="K39" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="L39" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="M39" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="N39" s="6">
+        <v>10</v>
+      </c>
+      <c r="O39" s="6">
+        <v>10</v>
+      </c>
+      <c r="P39" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="R39" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S39" s="7" t="s">
+        <v>1046</v>
+      </c>
+      <c r="T39" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="U39" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V39" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W39" s="7" t="s">
+        <v>1047</v>
+      </c>
+      <c r="X39" s="7" t="s">
+        <v>1048</v>
+      </c>
+      <c r="Y39" s="7" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="G40" s="5">
+        <v>6</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>918</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="J40" s="2">
+        <v>4</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="L40" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M40" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="N40" s="2">
+        <v>3</v>
+      </c>
+      <c r="O40" s="2">
+        <v>3</v>
+      </c>
+      <c r="P40" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="R40" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S40" s="3" t="s">
+        <v>1050</v>
+      </c>
+      <c r="T40" s="3" t="s">
+        <v>713</v>
+      </c>
+      <c r="U40" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V40" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="W40" s="3" t="s">
+        <v>1051</v>
+      </c>
+      <c r="X40" s="3" t="s">
+        <v>1052</v>
+      </c>
+      <c r="Y40" s="3" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="G41" s="9">
+        <v>7</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="J41" s="6">
+        <v>6</v>
+      </c>
+      <c r="K41" s="7" t="s">
+        <v>479</v>
+      </c>
+      <c r="L41" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="M41" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="N41" s="6">
+        <v>5</v>
+      </c>
+      <c r="O41" s="6">
+        <v>5</v>
+      </c>
+      <c r="P41" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="R41" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S41" s="7" t="s">
+        <v>1054</v>
+      </c>
+      <c r="T41" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="U41" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="V41" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="W41" s="7" t="s">
+        <v>1055</v>
+      </c>
+      <c r="X41" s="7" t="s">
+        <v>1056</v>
+      </c>
+      <c r="Y41" s="7" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Y1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>